<commit_message>
starting to diverge from our ealier handwritten code and converge using the most update esp libraries the first step to eliminate our custom console crate and using the original esp-println this refactoring can't happen in one step, so we try to reach at least a buildable version
</commit_message>
<xml_diff>
--- a/studies/ecu-via-elm327/sizing.xlsx
+++ b/studies/ecu-via-elm327/sizing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/piv/esp/ccm-diag/studies/ecu-via-elm327/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B268B18-0BD8-FA4C-B329-81836E86B81A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6546CABF-ECE8-534B-8B36-3A424378893E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="80" yWindow="500" windowWidth="25520" windowHeight="14900" xr2:uid="{7B075F7D-2CA4-8A4E-BD0B-AF2636EE3FAE}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2960" uniqueCount="2580">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2971" uniqueCount="2591">
   <si>
     <t>.bss</t>
   </si>
@@ -7652,9 +7652,6 @@
     <t>3FC87438</t>
   </si>
   <si>
-    <t>3FC887b8</t>
-  </si>
-  <si>
     <t>ecu_via_elm327::ecu::server::POOL</t>
   </si>
   <si>
@@ -7791,6 +7788,42 @@
   </si>
   <si>
     <t>all data</t>
+  </si>
+  <si>
+    <t>3FC887b0</t>
+  </si>
+  <si>
+    <t>----</t>
+  </si>
+  <si>
+    <t>---</t>
+  </si>
+  <si>
+    <t>-----</t>
+  </si>
+  <si>
+    <t>x----</t>
+  </si>
+  <si>
+    <t>x--2374</t>
+  </si>
+  <si>
+    <t>x++1062</t>
+  </si>
+  <si>
+    <t>x--54</t>
+  </si>
+  <si>
+    <t>x++36d4</t>
+  </si>
+  <si>
+    <t>x++66d2</t>
+  </si>
+  <si>
+    <t>x--5b8</t>
+  </si>
+  <si>
+    <t>x++3304</t>
   </si>
 </sst>
 </file>
@@ -7902,7 +7935,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -7946,6 +7979,7 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8372,9 +8406,6 @@
         <f t="shared" si="0"/>
         <v>0x1190</v>
       </c>
-      <c r="D5" t="s">
-        <v>2510</v>
-      </c>
       <c r="F5" t="s">
         <v>2531</v>
       </c>
@@ -8393,9 +8424,6 @@
       <c r="C6" s="10" t="str">
         <f t="shared" si="0"/>
         <v>0x1EC</v>
-      </c>
-      <c r="D6" t="s">
-        <v>2510</v>
       </c>
       <c r="G6" s="21">
         <f>B1+B2+B3</f>
@@ -8466,9 +8494,6 @@
         <f t="shared" si="0"/>
         <v>0x66D0</v>
       </c>
-      <c r="D9" t="s">
-        <v>2510</v>
-      </c>
       <c r="F9" t="s">
         <v>2511</v>
       </c>
@@ -8546,7 +8571,9 @@
         <f>B1+B2+B12+B13</f>
         <v>2562</v>
       </c>
-      <c r="E13" s="6"/>
+      <c r="E13" s="6" t="s">
+        <v>2583</v>
+      </c>
       <c r="F13" t="s">
         <v>2385</v>
       </c>
@@ -8567,7 +8594,9 @@
         <f>B14</f>
         <v>9184</v>
       </c>
-      <c r="E14" s="6"/>
+      <c r="E14" s="6" t="s">
+        <v>2584</v>
+      </c>
       <c r="F14" t="s">
         <v>2386</v>
       </c>
@@ -8584,6 +8613,9 @@
         <f t="shared" si="1"/>
         <v>0x1024</v>
       </c>
+      <c r="E15" t="s">
+        <v>2585</v>
+      </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -8635,7 +8667,9 @@
         <f>B17+B18</f>
         <v>2032</v>
       </c>
-      <c r="E18" s="6"/>
+      <c r="E18" s="6" t="s">
+        <v>2586</v>
+      </c>
       <c r="F18" t="s">
         <v>2388</v>
       </c>
@@ -8656,7 +8690,9 @@
         <f>B19</f>
         <v>13808</v>
       </c>
-      <c r="E19" s="6"/>
+      <c r="E19" s="6" t="s">
+        <v>2587</v>
+      </c>
       <c r="F19" t="s">
         <v>2389</v>
       </c>
@@ -8730,7 +8766,7 @@
         <v>341020</v>
       </c>
       <c r="H24" s="21" t="s">
-        <v>2578</v>
+        <v>2577</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
@@ -8758,7 +8794,7 @@
         <v>45004</v>
       </c>
       <c r="H25" s="21" t="s">
-        <v>2579</v>
+        <v>2578</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
@@ -8777,7 +8813,9 @@
         <f>B26</f>
         <v>26398</v>
       </c>
-      <c r="E26" s="6"/>
+      <c r="E26" s="6" t="s">
+        <v>2588</v>
+      </c>
       <c r="F26" t="s">
         <v>2391</v>
       </c>
@@ -8798,6 +8836,12 @@
         <f t="shared" si="1"/>
         <v>0x64A</v>
       </c>
+      <c r="D27" t="s">
+        <v>2510</v>
+      </c>
+      <c r="E27" t="s">
+        <v>2589</v>
+      </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
@@ -8810,6 +8854,12 @@
       <c r="C28" s="10" t="str">
         <f t="shared" si="1"/>
         <v>0x2EFE</v>
+      </c>
+      <c r="D28" t="s">
+        <v>2510</v>
+      </c>
+      <c r="E28" t="s">
+        <v>2590</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
@@ -8946,7 +8996,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>2552</v>
+        <v>2551</v>
       </c>
       <c r="B13">
         <v>224</v>
@@ -8986,7 +9036,7 @@
         <v>0x42014298</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>718</v>
       </c>
@@ -8998,13 +9048,13 @@
         <v>0x42014300</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C18" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B17))</f>
         <v>0x42014334</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>2459</v>
       </c>
@@ -9016,7 +9066,7 @@
         <v>0x42014334</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>720</v>
       </c>
@@ -9028,7 +9078,7 @@
         <v>0x420143DE</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>721</v>
       </c>
@@ -9040,7 +9090,7 @@
         <v>0x4201450E</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>719</v>
       </c>
@@ -9052,13 +9102,13 @@
         <v>0x42014604</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C23" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B22))</f>
         <v>0x42014618</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>722</v>
       </c>
@@ -9070,7 +9120,7 @@
         <v>0x42014618</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>723</v>
       </c>
@@ -9082,7 +9132,7 @@
         <v>0x4201461A</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>724</v>
       </c>
@@ -9094,7 +9144,7 @@
         <v>0x42014636</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>725</v>
       </c>
@@ -9106,7 +9156,7 @@
         <v>0x42014638</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>726</v>
       </c>
@@ -9118,7 +9168,7 @@
         <v>0x4201464C</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>727</v>
       </c>
@@ -9129,8 +9179,11 @@
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B28))</f>
         <v>0x420146D6</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D29" s="25" t="s">
+        <v>2581</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>728</v>
       </c>
@@ -9141,8 +9194,11 @@
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B29))</f>
         <v>0x420146DE</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D30" s="25" t="s">
+        <v>2580</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>729</v>
       </c>
@@ -9154,7 +9210,7 @@
         <v>0x420146E6</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>730</v>
       </c>
@@ -9166,13 +9222,13 @@
         <v>0x42014752</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C33" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B32))</f>
         <v>0x42014798</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>731</v>
       </c>
@@ -9184,9 +9240,9 @@
         <v>0x42014798</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>2565</v>
+        <v>2564</v>
       </c>
       <c r="B35">
         <v>206</v>
@@ -9196,9 +9252,9 @@
         <v>0x42014864</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>2566</v>
+        <v>2565</v>
       </c>
       <c r="B36">
         <v>200</v>
@@ -9208,13 +9264,13 @@
         <v>0x42014932</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C37" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B36))</f>
         <v>0x420149FA</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>732</v>
       </c>
@@ -9225,8 +9281,11 @@
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B37))</f>
         <v>0x420149FA</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D38">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>732</v>
       </c>
@@ -9238,7 +9297,7 @@
         <v>0x42014AA8</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>2401</v>
       </c>
@@ -9249,8 +9308,11 @@
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B39))</f>
         <v>0x42014AB0</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D40">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>733</v>
       </c>
@@ -9261,8 +9323,11 @@
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B40))</f>
         <v>0x42014B64</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D41">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>734</v>
       </c>
@@ -9274,7 +9339,7 @@
         <v>0x42014C24</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>2460</v>
       </c>
@@ -9286,7 +9351,7 @@
         <v>0x42014C90</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>735</v>
       </c>
@@ -9295,7 +9360,7 @@
         <v>0x42014E00</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>736</v>
       </c>
@@ -9307,13 +9372,13 @@
         <v>0x42014E00</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C46" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B45))</f>
         <v>0x42014F46</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>737</v>
       </c>
@@ -9325,7 +9390,7 @@
         <v>0x42014F46</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>738</v>
       </c>
@@ -9337,13 +9402,13 @@
         <v>0x42014F5A</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C49" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B48))</f>
         <v>0x42015082</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>739</v>
       </c>
@@ -9354,8 +9419,11 @@
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B49))</f>
         <v>0x42015082</v>
       </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D50">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>2464</v>
       </c>
@@ -9367,13 +9435,13 @@
         <v>0x4201522E</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C52" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B51))</f>
         <v>0x42015290</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>740</v>
       </c>
@@ -9385,7 +9453,7 @@
         <v>0x42015290</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>741</v>
       </c>
@@ -9397,7 +9465,7 @@
         <v>0x420152BE</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>742</v>
       </c>
@@ -9409,7 +9477,7 @@
         <v>0x420152CE</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>2402</v>
       </c>
@@ -9418,7 +9486,7 @@
         <v>0x420152DE</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>743</v>
       </c>
@@ -9430,7 +9498,7 @@
         <v>0x420152DE</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>744</v>
       </c>
@@ -9442,7 +9510,7 @@
         <v>0x4201532C</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>745</v>
       </c>
@@ -9454,7 +9522,7 @@
         <v>0x42015366</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>746</v>
       </c>
@@ -9466,7 +9534,7 @@
         <v>0x4201536E</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>747</v>
       </c>
@@ -9478,7 +9546,7 @@
         <v>0x420153B0</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>748</v>
       </c>
@@ -9490,7 +9558,7 @@
         <v>0x420153CA</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>749</v>
       </c>
@@ -9502,7 +9570,7 @@
         <v>0x420153EC</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>750</v>
       </c>
@@ -9682,7 +9750,7 @@
         <v>0x420155F0</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>765</v>
       </c>
@@ -9694,7 +9762,7 @@
         <v>0x42015638</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>766</v>
       </c>
@@ -9706,7 +9774,7 @@
         <v>0x420156D8</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>767</v>
       </c>
@@ -9718,7 +9786,7 @@
         <v>0x42015708</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>770</v>
       </c>
@@ -9729,8 +9797,11 @@
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B83))</f>
         <v>0x4201570C</v>
       </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D84">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>771</v>
       </c>
@@ -9742,7 +9813,7 @@
         <v>0x4201575A</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>772</v>
       </c>
@@ -9754,7 +9825,7 @@
         <v>0x4201575E</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>773</v>
       </c>
@@ -9766,7 +9837,7 @@
         <v>0x42015760</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>774</v>
       </c>
@@ -9778,7 +9849,7 @@
         <v>0x42015764</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>775</v>
       </c>
@@ -9790,7 +9861,7 @@
         <v>0x42015766</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>776</v>
       </c>
@@ -9802,7 +9873,7 @@
         <v>0x4201576A</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>777</v>
       </c>
@@ -9814,7 +9885,7 @@
         <v>0x4201576E</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>778</v>
       </c>
@@ -9826,7 +9897,7 @@
         <v>0x42015772</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>779</v>
       </c>
@@ -9838,7 +9909,7 @@
         <v>0x42015776</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>780</v>
       </c>
@@ -9850,7 +9921,7 @@
         <v>0x4201577A</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>781</v>
       </c>
@@ -9862,7 +9933,7 @@
         <v>0x4201577C</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>782</v>
       </c>
@@ -9874,7 +9945,7 @@
         <v>0x42015780</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>783</v>
       </c>
@@ -9886,7 +9957,7 @@
         <v>0x42015784</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>784</v>
       </c>
@@ -9898,7 +9969,7 @@
         <v>0x4201578C</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>2410</v>
       </c>
@@ -9907,7 +9978,7 @@
         <v>0x4201579C</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>785</v>
       </c>
@@ -9919,7 +9990,7 @@
         <v>0x4201579C</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>786</v>
       </c>
@@ -9930,8 +10001,11 @@
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B100))</f>
         <v>0x420157AA</v>
       </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D101">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>787</v>
       </c>
@@ -9943,7 +10017,7 @@
         <v>0x42015AD4</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>788</v>
       </c>
@@ -9955,7 +10029,7 @@
         <v>0x42015ADC</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>789</v>
       </c>
@@ -9967,24 +10041,24 @@
         <v>0x42015AE4</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C105" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B104))</f>
         <v>0x42015B2C</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>2567</v>
+        <v>2566</v>
       </c>
       <c r="C106" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B105))</f>
         <v>0x42015B2C</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>2568</v>
+        <v>2567</v>
       </c>
       <c r="B107">
         <v>40</v>
@@ -9993,14 +10067,17 @@
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B106))</f>
         <v>0x42015B2C</v>
       </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D107" s="25" t="s">
+        <v>2582</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C108" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B107))</f>
         <v>0x42015B54</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>2462</v>
       </c>
@@ -10012,7 +10089,7 @@
         <v>0x42015B54</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>1345</v>
       </c>
@@ -10024,7 +10101,7 @@
         <v>0x42015B5C</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>1837</v>
       </c>
@@ -10036,13 +10113,13 @@
         <v>0x42015C80</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C112" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B111))</f>
         <v>0x42015D0E</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>790</v>
       </c>
@@ -10053,8 +10130,11 @@
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B112))</f>
         <v>0x42015D0E</v>
       </c>
-    </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D113">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>791</v>
       </c>
@@ -10066,7 +10146,7 @@
         <v>0x42015DF0</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>792</v>
       </c>
@@ -10078,7 +10158,7 @@
         <v>0x42015F2E</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>793</v>
       </c>
@@ -10089,8 +10169,11 @@
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B115))</f>
         <v>0x42016080</v>
       </c>
-    </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D116">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>794</v>
       </c>
@@ -10101,14 +10184,17 @@
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B116))</f>
         <v>0x42016196</v>
       </c>
-    </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D117">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C118" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B117))</f>
         <v>0x42016322</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>795</v>
       </c>
@@ -10119,8 +10205,11 @@
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B118))</f>
         <v>0x42016322</v>
       </c>
-    </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D119">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>796</v>
       </c>
@@ -10132,13 +10221,13 @@
         <v>0x42016468</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C121" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B120))</f>
         <v>0x4201647A</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>797</v>
       </c>
@@ -10150,7 +10239,7 @@
         <v>0x4201647A</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>2405</v>
       </c>
@@ -10159,7 +10248,7 @@
         <v>0x42016658</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>2404</v>
       </c>
@@ -10170,8 +10259,11 @@
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B123))</f>
         <v>0x42016658</v>
       </c>
-    </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D124">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>2406</v>
       </c>
@@ -10180,7 +10272,7 @@
         <v>0x42016874</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>2404</v>
       </c>
@@ -10192,7 +10284,7 @@
         <v>0x42016874</v>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>798</v>
       </c>
@@ -10201,7 +10293,7 @@
         <v>0x42016A12</v>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>2409</v>
       </c>
@@ -10213,7 +10305,7 @@
         <v>0x42016A12</v>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>798</v>
       </c>
@@ -10222,7 +10314,7 @@
         <v>0x42016B7A</v>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>799</v>
       </c>
@@ -10234,7 +10326,7 @@
         <v>0x42016B7A</v>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>798</v>
       </c>
@@ -10243,7 +10335,7 @@
         <v>0x42016C4E</v>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>2407</v>
       </c>
@@ -10255,7 +10347,7 @@
         <v>0x42016C4E</v>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>798</v>
       </c>
@@ -10264,7 +10356,7 @@
         <v>0x42016F18</v>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>2408</v>
       </c>
@@ -10276,7 +10368,7 @@
         <v>0x42016F18</v>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>2419</v>
       </c>
@@ -10285,7 +10377,7 @@
         <v>0x42017000</v>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>800</v>
       </c>
@@ -10297,7 +10389,7 @@
         <v>0x42017000</v>
       </c>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>801</v>
       </c>
@@ -10309,7 +10401,7 @@
         <v>0x420170C4</v>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>802</v>
       </c>
@@ -10320,8 +10412,11 @@
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B137))</f>
         <v>0x420170EE</v>
       </c>
-    </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D138">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>803</v>
       </c>
@@ -10332,8 +10427,11 @@
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B138))</f>
         <v>0x42017188</v>
       </c>
-    </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D139">
+        <v>1188</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>2463</v>
       </c>
@@ -10345,13 +10443,13 @@
         <v>0x42017630</v>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C141" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B140))</f>
         <v>0x4201763A</v>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>804</v>
       </c>
@@ -10360,7 +10458,7 @@
         <v>0x4201763A</v>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>805</v>
       </c>
@@ -10372,7 +10470,7 @@
         <v>0x4201763A</v>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C144" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B143))</f>
         <v>0x42017650</v>
@@ -28458,7 +28556,7 @@
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>2564</v>
+        <v>2563</v>
       </c>
       <c r="B2">
         <v>294</v>
@@ -28739,7 +28837,7 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>2569</v>
+        <v>2568</v>
       </c>
       <c r="B26">
         <v>486</v>
@@ -28865,7 +28963,7 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>2570</v>
+        <v>2569</v>
       </c>
       <c r="B37">
         <v>398</v>
@@ -28943,7 +29041,7 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>2553</v>
+        <v>2552</v>
       </c>
       <c r="B44">
         <v>182</v>
@@ -29276,7 +29374,7 @@
         <v>24</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>2575</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -29434,7 +29532,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
-        <v>2554</v>
+        <v>2553</v>
       </c>
       <c r="D18" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C17))</f>
@@ -29443,7 +29541,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
-        <v>2555</v>
+        <v>2554</v>
       </c>
       <c r="C19">
         <v>2</v>
@@ -29461,7 +29559,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
-        <v>2556</v>
+        <v>2555</v>
       </c>
       <c r="C21">
         <f>11*62+20</f>
@@ -29472,7 +29570,7 @@
         <v>0x42058E44</v>
       </c>
       <c r="F21" t="s">
-        <v>2576</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
@@ -29481,12 +29579,12 @@
         <v>0x42059102</v>
       </c>
       <c r="F22" t="s">
-        <v>2577</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
       <c r="C23">
         <v>2</v>
@@ -29539,6 +29637,9 @@
       <c r="C29">
         <v>1924</v>
       </c>
+      <c r="D29" s="10">
+        <v>1952</v>
+      </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
@@ -29547,6 +29648,9 @@
       <c r="C30">
         <v>6764</v>
       </c>
+      <c r="D30" s="10">
+        <v>6908</v>
+      </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
@@ -29555,6 +29659,9 @@
       <c r="C31">
         <v>146</v>
       </c>
+      <c r="D31" s="10">
+        <v>212</v>
+      </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
@@ -29571,15 +29678,18 @@
       <c r="C33">
         <v>1398</v>
       </c>
+      <c r="D33" s="10">
+        <v>1412</v>
+      </c>
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B35" t="s">
-        <v>2558</v>
+        <v>2557</v>
       </c>
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B36" t="s">
-        <v>2559</v>
+        <v>2558</v>
       </c>
       <c r="C36">
         <v>464</v>
@@ -29587,12 +29697,12 @@
     </row>
     <row r="37" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B37" t="s">
-        <v>2558</v>
+        <v>2557</v>
       </c>
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B38" t="s">
-        <v>2560</v>
+        <v>2559</v>
       </c>
       <c r="C38">
         <v>312</v>
@@ -29600,12 +29710,12 @@
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B39" t="s">
-        <v>2558</v>
+        <v>2557</v>
       </c>
     </row>
     <row r="40" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B40" t="s">
-        <v>2561</v>
+        <v>2560</v>
       </c>
       <c r="C40">
         <v>282</v>
@@ -29613,7 +29723,7 @@
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B41" t="s">
-        <v>2562</v>
+        <v>2561</v>
       </c>
       <c r="C41">
         <v>314</v>
@@ -29621,7 +29731,7 @@
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B42" t="s">
-        <v>2563</v>
+        <v>2562</v>
       </c>
       <c r="C42">
         <v>300</v>
@@ -29629,7 +29739,7 @@
     </row>
     <row r="44" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B44" t="s">
-        <v>2572</v>
+        <v>2571</v>
       </c>
       <c r="C44">
         <v>2</v>
@@ -34247,7 +34357,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>2533</v>
+        <v>2579</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -34259,7 +34369,7 @@
       </c>
       <c r="C3" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B2))</f>
-        <v>0x3FC887BC</v>
+        <v>0x3FC887B4</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -34271,7 +34381,7 @@
       </c>
       <c r="C4" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B3))</f>
-        <v>0x3FC887C0</v>
+        <v>0x3FC887B8</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -34283,7 +34393,7 @@
       </c>
       <c r="C5" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B4))</f>
-        <v>0x3FC887C1</v>
+        <v>0x3FC887B9</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -34295,7 +34405,7 @@
       </c>
       <c r="C6" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B5))</f>
-        <v>0x3FC887C4</v>
+        <v>0x3FC887BC</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -34307,7 +34417,7 @@
       </c>
       <c r="C7" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B6))</f>
-        <v>0x3FC887C8</v>
+        <v>0x3FC887C0</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -34319,7 +34429,7 @@
       </c>
       <c r="C8" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B7))</f>
-        <v>0x3FC887CC</v>
+        <v>0x3FC887C4</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -34331,7 +34441,7 @@
       </c>
       <c r="C9" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B8))</f>
-        <v>0x3FC887D0</v>
+        <v>0x3FC887C8</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -34343,109 +34453,109 @@
       </c>
       <c r="C10" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B9))</f>
-        <v>0x3FC887D4</v>
+        <v>0x3FC887CC</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="C11" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B10))</f>
-        <v>0x3FC887D8</v>
+        <v>0x3FC887D0</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>2534</v>
+        <v>2533</v>
       </c>
       <c r="B12">
         <v>392</v>
       </c>
       <c r="C12" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B11))</f>
-        <v>0x3FC887D8</v>
+        <v>0x3FC887D0</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>2535</v>
+        <v>2534</v>
       </c>
       <c r="B13">
         <v>824</v>
       </c>
       <c r="C13" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B12))</f>
-        <v>0x3FC88960</v>
+        <v>0x3FC88958</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>2536</v>
+        <v>2535</v>
       </c>
       <c r="B14">
         <v>40</v>
       </c>
       <c r="C14" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B13))</f>
-        <v>0x3FC88C98</v>
+        <v>0x3FC88C90</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>2537</v>
+        <v>2536</v>
       </c>
       <c r="B15">
         <v>56</v>
       </c>
       <c r="C15" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B14))</f>
-        <v>0x3FC88CC0</v>
+        <v>0x3FC88CB8</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>2538</v>
+        <v>2537</v>
       </c>
       <c r="B16">
         <v>72</v>
       </c>
       <c r="C16" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B15))</f>
-        <v>0x3FC88CF8</v>
+        <v>0x3FC88CF0</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>2539</v>
+        <v>2538</v>
       </c>
       <c r="B17">
         <v>2</v>
       </c>
       <c r="C17" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B16))</f>
-        <v>0x3FC88D40</v>
+        <v>0x3FC88D38</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>2540</v>
+        <v>2539</v>
       </c>
       <c r="B18">
         <v>98304</v>
       </c>
       <c r="C18" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B17))</f>
-        <v>0x3FC88D42</v>
+        <v>0x3FC88D3A</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>2541</v>
+        <v>2540</v>
       </c>
       <c r="B19">
         <v>1</v>
       </c>
       <c r="C19" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B18))</f>
-        <v>0x3FCA0D42</v>
+        <v>0x3FCA0D3A</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
@@ -34457,67 +34567,67 @@
       </c>
       <c r="C20" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B19))</f>
-        <v>0x3FCA0D43</v>
+        <v>0x3FCA0D3B</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>2541</v>
+        <v>2540</v>
       </c>
       <c r="B21">
         <v>776</v>
       </c>
       <c r="C21" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B20))</f>
-        <v>0x3FCA0D48</v>
+        <v>0x3FCA0D40</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>2541</v>
+        <v>2540</v>
       </c>
       <c r="B22">
         <v>68</v>
       </c>
       <c r="C22" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B21))</f>
-        <v>0x3FCA1050</v>
+        <v>0x3FCA1048</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>2541</v>
+        <v>2540</v>
       </c>
       <c r="B23">
         <v>44</v>
       </c>
       <c r="C23" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B22))</f>
-        <v>0x3FCA1094</v>
+        <v>0x3FCA108C</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>2541</v>
+        <v>2540</v>
       </c>
       <c r="B24">
         <v>68</v>
       </c>
       <c r="C24" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B23))</f>
-        <v>0x3FCA10C0</v>
+        <v>0x3FCA10B8</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>2541</v>
+        <v>2540</v>
       </c>
       <c r="B25">
         <v>44</v>
       </c>
       <c r="C25" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B24))</f>
-        <v>0x3FCA1104</v>
+        <v>0x3FCA10FC</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
@@ -34529,7 +34639,7 @@
       </c>
       <c r="C26" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B25))</f>
-        <v>0x3FCA1130</v>
+        <v>0x3FCA1128</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
@@ -34541,7 +34651,7 @@
       </c>
       <c r="C27" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B26))</f>
-        <v>0x3FCA1704</v>
+        <v>0x3FCA16FC</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
@@ -34553,7 +34663,7 @@
       </c>
       <c r="C28" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B27))</f>
-        <v>0x3FCA1708</v>
+        <v>0x3FCA1700</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
@@ -34565,7 +34675,7 @@
       </c>
       <c r="C29" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B28))</f>
-        <v>0x3FCA1714</v>
+        <v>0x3FCA170C</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
@@ -34577,7 +34687,7 @@
       </c>
       <c r="C30" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B29))</f>
-        <v>0x3FCA1768</v>
+        <v>0x3FCA1760</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
@@ -34589,7 +34699,7 @@
       </c>
       <c r="C31" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B30))</f>
-        <v>0x3FCA176C</v>
+        <v>0x3FCA1764</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
@@ -34601,7 +34711,7 @@
       </c>
       <c r="C32" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B31))</f>
-        <v>0x3FCA1778</v>
+        <v>0x3FCA1770</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
@@ -34613,7 +34723,7 @@
       </c>
       <c r="C33" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B32))</f>
-        <v>0x3FCA1784</v>
+        <v>0x3FCA177C</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
@@ -34625,7 +34735,7 @@
       </c>
       <c r="C34" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B33))</f>
-        <v>0x3FCA1790</v>
+        <v>0x3FCA1788</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
@@ -34637,7 +34747,7 @@
       </c>
       <c r="C35" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B34))</f>
-        <v>0x3FCA179C</v>
+        <v>0x3FCA1794</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
@@ -34649,7 +34759,7 @@
       </c>
       <c r="C36" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B35))</f>
-        <v>0x3FCA17A8</v>
+        <v>0x3FCA17A0</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
@@ -34661,7 +34771,7 @@
       </c>
       <c r="C37" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B36))</f>
-        <v>0x3FCA17B4</v>
+        <v>0x3FCA17AC</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
@@ -34673,7 +34783,7 @@
       </c>
       <c r="C38" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B37))</f>
-        <v>0x3FCA17B5</v>
+        <v>0x3FCA17AD</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
@@ -34685,7 +34795,7 @@
       </c>
       <c r="C39" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B38))</f>
-        <v>0x3FCA17B8</v>
+        <v>0x3FCA17B0</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
@@ -34697,7 +34807,7 @@
       </c>
       <c r="C40" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B39))</f>
-        <v>0x3FCA17BC</v>
+        <v>0x3FCA17B4</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
@@ -34709,7 +34819,7 @@
       </c>
       <c r="C41" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B40))</f>
-        <v>0x3FCA17C0</v>
+        <v>0x3FCA17B8</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
@@ -34721,7 +34831,7 @@
       </c>
       <c r="C42" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B41))</f>
-        <v>0x3FCA17C4</v>
+        <v>0x3FCA17BC</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
@@ -34733,7 +34843,7 @@
       </c>
       <c r="C43" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B42))</f>
-        <v>0x3FCA17C5</v>
+        <v>0x3FCA17BD</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
@@ -34745,7 +34855,7 @@
       </c>
       <c r="C44" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B43))</f>
-        <v>0x3FCA17C8</v>
+        <v>0x3FCA17C0</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
@@ -34757,7 +34867,7 @@
       </c>
       <c r="C45" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B44))</f>
-        <v>0x3FCA17E0</v>
+        <v>0x3FCA17D8</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
@@ -34769,7 +34879,7 @@
       </c>
       <c r="C46" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B45))</f>
-        <v>0x3FCA17E1</v>
+        <v>0x3FCA17D9</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
@@ -34781,7 +34891,7 @@
       </c>
       <c r="C47" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B46))</f>
-        <v>0x3FCA17E4</v>
+        <v>0x3FCA17DC</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
@@ -34793,7 +34903,7 @@
       </c>
       <c r="C48" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B47))</f>
-        <v>0x3FCA17E8</v>
+        <v>0x3FCA17E0</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
@@ -34805,7 +34915,7 @@
       </c>
       <c r="C49" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B48))</f>
-        <v>0x3FCA17EC</v>
+        <v>0x3FCA17E4</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
@@ -34817,7 +34927,7 @@
       </c>
       <c r="C50" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B49))</f>
-        <v>0x3FCA17F4</v>
+        <v>0x3FCA17EC</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
@@ -34829,7 +34939,7 @@
       </c>
       <c r="C51" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B50))</f>
-        <v>0x3FCA1800</v>
+        <v>0x3FCA17F8</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
@@ -34841,7 +34951,7 @@
       </c>
       <c r="C52" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B51))</f>
-        <v>0x3FCA180C</v>
+        <v>0x3FCA1804</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
@@ -34853,7 +34963,7 @@
       </c>
       <c r="C53" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B52))</f>
-        <v>0x3FCA1818</v>
+        <v>0x3FCA1810</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
@@ -34865,7 +34975,7 @@
       </c>
       <c r="C54" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B53))</f>
-        <v>0x3FCA1824</v>
+        <v>0x3FCA181C</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
@@ -34877,7 +34987,7 @@
       </c>
       <c r="C55" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B54))</f>
-        <v>0x3FCA1830</v>
+        <v>0x3FCA1828</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
@@ -34889,7 +34999,7 @@
       </c>
       <c r="C56" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B55))</f>
-        <v>0x3FCA183C</v>
+        <v>0x3FCA1834</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
@@ -34901,7 +35011,7 @@
       </c>
       <c r="C57" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B56))</f>
-        <v>0x3FCA1848</v>
+        <v>0x3FCA1840</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
@@ -34913,7 +35023,7 @@
       </c>
       <c r="C58" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B57))</f>
-        <v>0x3FCA1854</v>
+        <v>0x3FCA184C</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
@@ -34925,7 +35035,7 @@
       </c>
       <c r="C59" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B58))</f>
-        <v>0x3FCA1860</v>
+        <v>0x3FCA1858</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
@@ -34937,7 +35047,7 @@
       </c>
       <c r="C60" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B59))</f>
-        <v>0x3FCA186C</v>
+        <v>0x3FCA1864</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.2">
@@ -34949,7 +35059,7 @@
       </c>
       <c r="C61" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B60))</f>
-        <v>0x3FCA1878</v>
+        <v>0x3FCA1870</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
@@ -34961,7 +35071,7 @@
       </c>
       <c r="C62" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B61))</f>
-        <v>0x3FCA1884</v>
+        <v>0x3FCA187C</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.2">
@@ -34973,7 +35083,7 @@
       </c>
       <c r="C63" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B62))</f>
-        <v>0x3FCA1890</v>
+        <v>0x3FCA1888</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.2">
@@ -34985,7 +35095,7 @@
       </c>
       <c r="C64" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B63))</f>
-        <v>0x3FCA189C</v>
+        <v>0x3FCA1894</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
@@ -34997,7 +35107,7 @@
       </c>
       <c r="C65" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B64))</f>
-        <v>0x3FCA18BC</v>
+        <v>0x3FCA18B4</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.2">
@@ -35009,7 +35119,7 @@
       </c>
       <c r="C66" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B65))</f>
-        <v>0x3FCA18BD</v>
+        <v>0x3FCA18B5</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.2">
@@ -35021,7 +35131,7 @@
       </c>
       <c r="C67" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B66))</f>
-        <v>0x3FCA18D5</v>
+        <v>0x3FCA18CD</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.2">
@@ -35033,7 +35143,7 @@
       </c>
       <c r="C68" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B67))</f>
-        <v>0x3FCA18D8</v>
+        <v>0x3FCA18D0</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.2">
@@ -35045,7 +35155,7 @@
       </c>
       <c r="C69" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B68))</f>
-        <v>0x3FCA18D9</v>
+        <v>0x3FCA18D1</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.2">
@@ -35057,7 +35167,7 @@
       </c>
       <c r="C70" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B69))</f>
-        <v>0x3FCA18DF</v>
+        <v>0x3FCA18D7</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
@@ -35069,7 +35179,7 @@
       </c>
       <c r="C71" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B70))</f>
-        <v>0x3FCA18E0</v>
+        <v>0x3FCA18D8</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
@@ -35081,7 +35191,7 @@
       </c>
       <c r="C72" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B71))</f>
-        <v>0x3FCA18E1</v>
+        <v>0x3FCA18D9</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.2">
@@ -35093,7 +35203,7 @@
       </c>
       <c r="C73" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B72))</f>
-        <v>0x3FCA18E4</v>
+        <v>0x3FCA18DC</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.2">
@@ -35105,7 +35215,7 @@
       </c>
       <c r="C74" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B73))</f>
-        <v>0x3FCA18F4</v>
+        <v>0x3FCA18EC</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
@@ -35117,7 +35227,7 @@
       </c>
       <c r="C75" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B74))</f>
-        <v>0x3FCA18F5</v>
+        <v>0x3FCA18ED</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.2">
@@ -35129,7 +35239,7 @@
       </c>
       <c r="C76" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B75))</f>
-        <v>0x3FCA18F6</v>
+        <v>0x3FCA18EE</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.2">
@@ -35141,7 +35251,7 @@
       </c>
       <c r="C77" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B76))</f>
-        <v>0x3FCA18F8</v>
+        <v>0x3FCA18F0</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.2">
@@ -35153,7 +35263,7 @@
       </c>
       <c r="C78" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B77))</f>
-        <v>0x3FCA18FC</v>
+        <v>0x3FCA18F4</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.2">
@@ -35165,7 +35275,7 @@
       </c>
       <c r="C79" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B78))</f>
-        <v>0x3FCA18FD</v>
+        <v>0x3FCA18F5</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.2">
@@ -35177,7 +35287,7 @@
       </c>
       <c r="C80" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B79))</f>
-        <v>0x3FCA1900</v>
+        <v>0x3FCA18F8</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.2">
@@ -35189,7 +35299,7 @@
       </c>
       <c r="C81" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B80))</f>
-        <v>0x3FCA1904</v>
+        <v>0x3FCA18FC</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.2">
@@ -35201,7 +35311,7 @@
       </c>
       <c r="C82" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B81))</f>
-        <v>0x3FCA1908</v>
+        <v>0x3FCA1900</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.2">
@@ -35213,7 +35323,7 @@
       </c>
       <c r="C83" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B82))</f>
-        <v>0x3FCA1909</v>
+        <v>0x3FCA1901</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.2">
@@ -35225,7 +35335,7 @@
       </c>
       <c r="C84" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B83))</f>
-        <v>0x3FCA190C</v>
+        <v>0x3FCA1904</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.2">
@@ -35237,7 +35347,7 @@
       </c>
       <c r="C85" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B84))</f>
-        <v>0x3FCA1BA8</v>
+        <v>0x3FCA1BA0</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.2">
@@ -35249,7 +35359,7 @@
       </c>
       <c r="C86" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B85))</f>
-        <v>0x3FCA1BAC</v>
+        <v>0x3FCA1BA4</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.2">
@@ -35261,7 +35371,7 @@
       </c>
       <c r="C87" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B86))</f>
-        <v>0x3FCA1BB0</v>
+        <v>0x3FCA1BA8</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.2">
@@ -35273,7 +35383,7 @@
       </c>
       <c r="C88" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B87))</f>
-        <v>0x3FCA1BB4</v>
+        <v>0x3FCA1BAC</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.2">
@@ -35285,7 +35395,7 @@
       </c>
       <c r="C89" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B88))</f>
-        <v>0x3FCA1C28</v>
+        <v>0x3FCA1C20</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.2">
@@ -35297,7 +35407,7 @@
       </c>
       <c r="C90" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B89))</f>
-        <v>0x3FCA1C68</v>
+        <v>0x3FCA1C60</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.2">
@@ -35309,7 +35419,7 @@
       </c>
       <c r="C91" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B90))</f>
-        <v>0x3FCA1C7C</v>
+        <v>0x3FCA1C74</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.2">
@@ -35321,7 +35431,7 @@
       </c>
       <c r="C92" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B91))</f>
-        <v>0x3FCA1C88</v>
+        <v>0x3FCA1C80</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.2">
@@ -35333,7 +35443,7 @@
       </c>
       <c r="C93" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B92))</f>
-        <v>0x3FCA1C9C</v>
+        <v>0x3FCA1C94</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.2">
@@ -35345,7 +35455,7 @@
       </c>
       <c r="C94" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B93))</f>
-        <v>0x3FCA1CA0</v>
+        <v>0x3FCA1C98</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.2">
@@ -35357,7 +35467,7 @@
       </c>
       <c r="C95" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B94))</f>
-        <v>0x3FCA1CA1</v>
+        <v>0x3FCA1C99</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.2">
@@ -35369,7 +35479,7 @@
       </c>
       <c r="C96" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B95))</f>
-        <v>0x3FCA1CA2</v>
+        <v>0x3FCA1C9A</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.2">
@@ -35381,7 +35491,7 @@
       </c>
       <c r="C97" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B96))</f>
-        <v>0x3FCA1CA4</v>
+        <v>0x3FCA1C9C</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.2">
@@ -35393,7 +35503,7 @@
       </c>
       <c r="C98" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B97))</f>
-        <v>0x3FCA1CA8</v>
+        <v>0x3FCA1CA0</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.2">
@@ -35405,7 +35515,7 @@
       </c>
       <c r="C99" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B98))</f>
-        <v>0x3FCA1CAC</v>
+        <v>0x3FCA1CA4</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.2">
@@ -35417,7 +35527,7 @@
       </c>
       <c r="C100" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B99))</f>
-        <v>0x3FCA1CB0</v>
+        <v>0x3FCA1CA8</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.2">
@@ -35429,7 +35539,7 @@
       </c>
       <c r="C101" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B100))</f>
-        <v>0x3FCA1CB4</v>
+        <v>0x3FCA1CAC</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.2">
@@ -35441,7 +35551,7 @@
       </c>
       <c r="C102" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B101))</f>
-        <v>0x3FCA1CB5</v>
+        <v>0x3FCA1CAD</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.2">
@@ -35453,7 +35563,7 @@
       </c>
       <c r="C103" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B102))</f>
-        <v>0x3FCA1CB8</v>
+        <v>0x3FCA1CB0</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.2">
@@ -35465,7 +35575,7 @@
       </c>
       <c r="C104" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B103))</f>
-        <v>0x3FCA1CCC</v>
+        <v>0x3FCA1CC4</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.2">
@@ -35477,7 +35587,7 @@
       </c>
       <c r="C105" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B104))</f>
-        <v>0x3FCA1CCD</v>
+        <v>0x3FCA1CC5</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.2">
@@ -35489,7 +35599,7 @@
       </c>
       <c r="C106" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B105))</f>
-        <v>0x3FCA1CD0</v>
+        <v>0x3FCA1CC8</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.2">
@@ -35501,7 +35611,7 @@
       </c>
       <c r="C107" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B106))</f>
-        <v>0x3FCA1CD8</v>
+        <v>0x3FCA1CD0</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.2">
@@ -35513,7 +35623,7 @@
       </c>
       <c r="C108" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B107))</f>
-        <v>0x3FCA1CD9</v>
+        <v>0x3FCA1CD1</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.2">
@@ -35525,7 +35635,7 @@
       </c>
       <c r="C109" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B108))</f>
-        <v>0x3FCA1CDA</v>
+        <v>0x3FCA1CD2</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.2">
@@ -35537,7 +35647,7 @@
       </c>
       <c r="C110" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B109))</f>
-        <v>0x3FCA1CDB</v>
+        <v>0x3FCA1CD3</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.2">
@@ -35549,7 +35659,7 @@
       </c>
       <c r="C111" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B110))</f>
-        <v>0x3FCA1CDC</v>
+        <v>0x3FCA1CD4</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.2">
@@ -35561,7 +35671,7 @@
       </c>
       <c r="C112" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B111))</f>
-        <v>0x3FCA1CE0</v>
+        <v>0x3FCA1CD8</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.2">
@@ -35573,7 +35683,7 @@
       </c>
       <c r="C113" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B112))</f>
-        <v>0x3FCA1CE1</v>
+        <v>0x3FCA1CD9</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.2">
@@ -35585,7 +35695,7 @@
       </c>
       <c r="C114" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B113))</f>
-        <v>0x3FCA1CE2</v>
+        <v>0x3FCA1CDA</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.2">
@@ -35597,7 +35707,7 @@
       </c>
       <c r="C115" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B114))</f>
-        <v>0x3FCA1CE8</v>
+        <v>0x3FCA1CE0</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.2">
@@ -35609,7 +35719,7 @@
       </c>
       <c r="C116" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B115))</f>
-        <v>0x3FCA1D50</v>
+        <v>0x3FCA1D48</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.2">
@@ -35621,7 +35731,7 @@
       </c>
       <c r="C117" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B116))</f>
-        <v>0x3FCA1D54</v>
+        <v>0x3FCA1D4C</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.2">
@@ -35633,7 +35743,7 @@
       </c>
       <c r="C118" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B117))</f>
-        <v>0x3FCA1D55</v>
+        <v>0x3FCA1D4D</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.2">
@@ -35645,7 +35755,7 @@
       </c>
       <c r="C119" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B118))</f>
-        <v>0x3FCA1D56</v>
+        <v>0x3FCA1D4E</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.2">
@@ -35657,7 +35767,7 @@
       </c>
       <c r="C120" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B119))</f>
-        <v>0x3FCA1D58</v>
+        <v>0x3FCA1D50</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.2">
@@ -35669,7 +35779,7 @@
       </c>
       <c r="C121" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B120))</f>
-        <v>0x3FCA1D5C</v>
+        <v>0x3FCA1D54</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.2">
@@ -35681,7 +35791,7 @@
       </c>
       <c r="C122" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B121))</f>
-        <v>0x3FCA1E0C</v>
+        <v>0x3FCA1E04</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.2">
@@ -35693,7 +35803,7 @@
       </c>
       <c r="C123" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B122))</f>
-        <v>0x3FCA1E10</v>
+        <v>0x3FCA1E08</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.2">
@@ -35705,7 +35815,7 @@
       </c>
       <c r="C124" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B123))</f>
-        <v>0x3FCA1E14</v>
+        <v>0x3FCA1E0C</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.2">
@@ -35717,7 +35827,7 @@
       </c>
       <c r="C125" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B124))</f>
-        <v>0x3FCA2318</v>
+        <v>0x3FCA2310</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.2">
@@ -35729,7 +35839,7 @@
       </c>
       <c r="C126" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B125))</f>
-        <v>0x3FCA2319</v>
+        <v>0x3FCA2311</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.2">
@@ -35741,7 +35851,7 @@
       </c>
       <c r="C127" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B126))</f>
-        <v>0x3FCA231C</v>
+        <v>0x3FCA2314</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.2">
@@ -35753,7 +35863,7 @@
       </c>
       <c r="C128" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B127))</f>
-        <v>0x3FCA2320</v>
+        <v>0x3FCA2318</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.2">
@@ -35765,7 +35875,7 @@
       </c>
       <c r="C129" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B128))</f>
-        <v>0x3FCA2328</v>
+        <v>0x3FCA2320</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.2">
@@ -35777,7 +35887,7 @@
       </c>
       <c r="C130" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B129))</f>
-        <v>0x3FCA2329</v>
+        <v>0x3FCA2321</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.2">
@@ -35789,7 +35899,7 @@
       </c>
       <c r="C131" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B130))</f>
-        <v>0x3FCA232C</v>
+        <v>0x3FCA2324</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.2">
@@ -35801,7 +35911,7 @@
       </c>
       <c r="C132" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B131))</f>
-        <v>0x3FCA233C</v>
+        <v>0x3FCA2334</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.2">
@@ -35813,7 +35923,7 @@
       </c>
       <c r="C133" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B132))</f>
-        <v>0x3FCA233D</v>
+        <v>0x3FCA2335</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.2">
@@ -35825,7 +35935,7 @@
       </c>
       <c r="C134" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B133))</f>
-        <v>0x3FCA2340</v>
+        <v>0x3FCA2338</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.2">
@@ -35837,7 +35947,7 @@
       </c>
       <c r="C135" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B134))</f>
-        <v>0x3FCA245C</v>
+        <v>0x3FCA2454</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.2">
@@ -35849,7 +35959,7 @@
       </c>
       <c r="C136" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B135))</f>
-        <v>0x3FCA245E</v>
+        <v>0x3FCA2456</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.2">
@@ -35861,7 +35971,7 @@
       </c>
       <c r="C137" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B136))</f>
-        <v>0x3FCA2460</v>
+        <v>0x3FCA2458</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.2">
@@ -35873,7 +35983,7 @@
       </c>
       <c r="C138" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B137))</f>
-        <v>0x3FCA2464</v>
+        <v>0x3FCA245C</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.2">
@@ -35885,7 +35995,7 @@
       </c>
       <c r="C139" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B138))</f>
-        <v>0x3FCA2466</v>
+        <v>0x3FCA245E</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.2">
@@ -35897,7 +36007,7 @@
       </c>
       <c r="C140" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B139))</f>
-        <v>0x3FCA2467</v>
+        <v>0x3FCA245F</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.2">
@@ -35909,7 +36019,7 @@
       </c>
       <c r="C141" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B140))</f>
-        <v>0x3FCA2468</v>
+        <v>0x3FCA2460</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.2">
@@ -35921,7 +36031,7 @@
       </c>
       <c r="C142" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B141))</f>
-        <v>0x3FCA2470</v>
+        <v>0x3FCA2468</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.2">
@@ -35933,7 +36043,7 @@
       </c>
       <c r="C143" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B142))</f>
-        <v>0x3FCA2474</v>
+        <v>0x3FCA246C</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.2">
@@ -35945,7 +36055,7 @@
       </c>
       <c r="C144" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B143))</f>
-        <v>0x3FCA2488</v>
+        <v>0x3FCA2480</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.2">
@@ -35957,7 +36067,7 @@
       </c>
       <c r="C145" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B144))</f>
-        <v>0x3FCA24D8</v>
+        <v>0x3FCA24D0</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.2">
@@ -35969,7 +36079,7 @@
       </c>
       <c r="C146" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B145))</f>
-        <v>0x3FCA2528</v>
+        <v>0x3FCA2520</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.2">
@@ -35981,7 +36091,7 @@
       </c>
       <c r="C147" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B146))</f>
-        <v>0x3FCA2750</v>
+        <v>0x3FCA2748</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.2">
@@ -35993,7 +36103,7 @@
       </c>
       <c r="C148" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B147))</f>
-        <v>0x3FCA2751</v>
+        <v>0x3FCA2749</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.2">
@@ -36005,7 +36115,7 @@
       </c>
       <c r="C149" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B148))</f>
-        <v>0x3FCA2754</v>
+        <v>0x3FCA274C</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.2">
@@ -36017,7 +36127,7 @@
       </c>
       <c r="C150" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B149))</f>
-        <v>0x3FCA2768</v>
+        <v>0x3FCA2760</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.2">
@@ -36029,7 +36139,7 @@
       </c>
       <c r="C151" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B150))</f>
-        <v>0x3FCA2769</v>
+        <v>0x3FCA2761</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.2">
@@ -36041,7 +36151,7 @@
       </c>
       <c r="C152" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B151))</f>
-        <v>0x3FCA276A</v>
+        <v>0x3FCA2762</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.2">
@@ -36053,7 +36163,7 @@
       </c>
       <c r="C153" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B152))</f>
-        <v>0x3FCA2770</v>
+        <v>0x3FCA2768</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.2">
@@ -36065,7 +36175,7 @@
       </c>
       <c r="C154" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B153))</f>
-        <v>0x3FCA3668</v>
+        <v>0x3FCA3660</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.2">
@@ -36077,7 +36187,7 @@
       </c>
       <c r="C155" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B154))</f>
-        <v>0x3FCA366C</v>
+        <v>0x3FCA3664</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.2">
@@ -36089,7 +36199,7 @@
       </c>
       <c r="C156" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B155))</f>
-        <v>0x3FCA366D</v>
+        <v>0x3FCA3665</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.2">
@@ -36101,7 +36211,7 @@
       </c>
       <c r="C157" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B156))</f>
-        <v>0x3FCA366E</v>
+        <v>0x3FCA3666</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.2">
@@ -36113,7 +36223,7 @@
       </c>
       <c r="C158" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B157))</f>
-        <v>0x3FCA366F</v>
+        <v>0x3FCA3667</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.2">
@@ -36125,7 +36235,7 @@
       </c>
       <c r="C159" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B158))</f>
-        <v>0x3FCA3670</v>
+        <v>0x3FCA3668</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.2">
@@ -36137,7 +36247,7 @@
       </c>
       <c r="C160" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B159))</f>
-        <v>0x3FCA3674</v>
+        <v>0x3FCA366C</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.2">
@@ -36149,7 +36259,7 @@
       </c>
       <c r="C161" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B160))</f>
-        <v>0x3FCA3676</v>
+        <v>0x3FCA366E</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.2">
@@ -36161,7 +36271,7 @@
       </c>
       <c r="C162" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B161))</f>
-        <v>0x3FCA3678</v>
+        <v>0x3FCA3670</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.2">
@@ -36173,13 +36283,13 @@
       </c>
       <c r="C163" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B162))</f>
-        <v>0x3FCA368C</v>
+        <v>0x3FCA3684</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.2">
       <c r="C164" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B163))</f>
-        <v>0x3FCA3694</v>
+        <v>0x3FCA368C</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.2">
@@ -36191,7 +36301,7 @@
       </c>
       <c r="C165" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B164))</f>
-        <v>0x3FCA3694</v>
+        <v>0x3FCA368C</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.2">
@@ -36203,7 +36313,7 @@
       </c>
       <c r="C166" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B165))</f>
-        <v>0x3FCA36BC</v>
+        <v>0x3FCA36B4</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.2">
@@ -36215,7 +36325,7 @@
       </c>
       <c r="C167" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B166))</f>
-        <v>0x3FCA36E6</v>
+        <v>0x3FCA36DE</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.2">
@@ -36227,7 +36337,7 @@
       </c>
       <c r="C168" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B167))</f>
-        <v>0x3FCA36E8</v>
+        <v>0x3FCA36E0</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.2">
@@ -36239,7 +36349,7 @@
       </c>
       <c r="C169" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B168))</f>
-        <v>0x3FCA36EC</v>
+        <v>0x3FCA36E4</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.2">
@@ -36251,7 +36361,7 @@
       </c>
       <c r="C170" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B169))</f>
-        <v>0x3FCA36ED</v>
+        <v>0x3FCA36E5</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.2">
@@ -36263,13 +36373,13 @@
       </c>
       <c r="C171" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B170))</f>
-        <v>0x3FCA36F0</v>
+        <v>0x3FCA36E8</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.2">
       <c r="C172" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B171))</f>
-        <v>0x3FCA36F4</v>
+        <v>0x3FCA36EC</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.2">
@@ -36281,7 +36391,7 @@
       </c>
       <c r="C173" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B172))</f>
-        <v>0x3FCA36F4</v>
+        <v>0x3FCA36EC</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.2">
@@ -36293,7 +36403,7 @@
       </c>
       <c r="C174" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B173))</f>
-        <v>0x3FCA37B4</v>
+        <v>0x3FCA37AC</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.2">
@@ -36305,7 +36415,7 @@
       </c>
       <c r="C175" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B174))</f>
-        <v>0x3FCA37DC</v>
+        <v>0x3FCA37D4</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.2">
@@ -36317,7 +36427,7 @@
       </c>
       <c r="C176" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B175))</f>
-        <v>0x3FCA37DD</v>
+        <v>0x3FCA37D5</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.2">
@@ -36329,7 +36439,7 @@
       </c>
       <c r="C177" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B176))</f>
-        <v>0x3FCA37E0</v>
+        <v>0x3FCA37D8</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.2">
@@ -36341,7 +36451,7 @@
       </c>
       <c r="C178" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B177))</f>
-        <v>0x3FCA37F4</v>
+        <v>0x3FCA37EC</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.2">
@@ -36353,7 +36463,7 @@
       </c>
       <c r="C179" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B178))</f>
-        <v>0x3FCA37F8</v>
+        <v>0x3FCA37F0</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.2">
@@ -36365,7 +36475,7 @@
       </c>
       <c r="C180" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B179))</f>
-        <v>0x3FCA3800</v>
+        <v>0x3FCA37F8</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.2">
@@ -36377,7 +36487,7 @@
       </c>
       <c r="C181" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B180))</f>
-        <v>0x3FCA39D0</v>
+        <v>0x3FCA39C8</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.2">
@@ -36389,7 +36499,7 @@
       </c>
       <c r="C182" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B181))</f>
-        <v>0x3FCA39D4</v>
+        <v>0x3FCA39CC</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.2">
@@ -36401,7 +36511,7 @@
       </c>
       <c r="C183" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B182))</f>
-        <v>0x3FCA39D8</v>
+        <v>0x3FCA39D0</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.2">
@@ -36413,7 +36523,7 @@
       </c>
       <c r="C184" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B183))</f>
-        <v>0x3FCA39E8</v>
+        <v>0x3FCA39E0</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.2">
@@ -36425,7 +36535,7 @@
       </c>
       <c r="C185" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B184))</f>
-        <v>0x3FCA3AA8</v>
+        <v>0x3FCA3AA0</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.2">
@@ -36437,7 +36547,7 @@
       </c>
       <c r="C186" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B185))</f>
-        <v>0x3FCA3AF0</v>
+        <v>0x3FCA3AE8</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.2">
@@ -36449,7 +36559,7 @@
       </c>
       <c r="C187" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B186))</f>
-        <v>0x3FCA3AF4</v>
+        <v>0x3FCA3AEC</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.2">
@@ -36461,7 +36571,7 @@
       </c>
       <c r="C188" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B187))</f>
-        <v>0x3FCA3AFC</v>
+        <v>0x3FCA3AF4</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.2">
@@ -36473,7 +36583,7 @@
       </c>
       <c r="C189" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B188))</f>
-        <v>0x3FCA3B00</v>
+        <v>0x3FCA3AF8</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.2">
@@ -36485,7 +36595,7 @@
       </c>
       <c r="C190" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B189))</f>
-        <v>0x3FCA3B04</v>
+        <v>0x3FCA3AFC</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.2">
@@ -36497,7 +36607,7 @@
       </c>
       <c r="C191" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B190))</f>
-        <v>0x3FCA3B08</v>
+        <v>0x3FCA3B00</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.2">
@@ -36509,7 +36619,7 @@
       </c>
       <c r="C192" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B191))</f>
-        <v>0x3FCA3B0C</v>
+        <v>0x3FCA3B04</v>
       </c>
     </row>
     <row r="193" spans="1:5" x14ac:dyDescent="0.2">
@@ -36521,7 +36631,7 @@
       </c>
       <c r="C193" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B192))</f>
-        <v>0x3FCA3B10</v>
+        <v>0x3FCA3B08</v>
       </c>
     </row>
     <row r="194" spans="1:5" x14ac:dyDescent="0.2">
@@ -36533,7 +36643,7 @@
       </c>
       <c r="C194" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B193))</f>
-        <v>0x3FCA3B14</v>
+        <v>0x3FCA3B0C</v>
       </c>
     </row>
     <row r="195" spans="1:5" x14ac:dyDescent="0.2">
@@ -36545,7 +36655,7 @@
       </c>
       <c r="C195" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B194))</f>
-        <v>0x3FCA3B18</v>
+        <v>0x3FCA3B10</v>
       </c>
     </row>
     <row r="196" spans="1:5" x14ac:dyDescent="0.2">
@@ -36557,7 +36667,7 @@
       </c>
       <c r="C196" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B195))</f>
-        <v>0x3FCA3B8C</v>
+        <v>0x3FCA3B84</v>
       </c>
     </row>
     <row r="197" spans="1:5" x14ac:dyDescent="0.2">
@@ -36569,13 +36679,13 @@
       </c>
       <c r="C197" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B196))</f>
-        <v>0x3FCA3B90</v>
+        <v>0x3FCA3B88</v>
       </c>
     </row>
     <row r="198" spans="1:5" x14ac:dyDescent="0.2">
       <c r="C198" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B197))</f>
-        <v>0x3FCA3B98</v>
+        <v>0x3FCA3B90</v>
       </c>
     </row>
     <row r="199" spans="1:5" x14ac:dyDescent="0.2">
@@ -36587,7 +36697,7 @@
       </c>
       <c r="C199" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B198))</f>
-        <v>0x3FCA3B98</v>
+        <v>0x3FCA3B90</v>
       </c>
     </row>
     <row r="200" spans="1:5" x14ac:dyDescent="0.2">
@@ -36599,7 +36709,7 @@
       </c>
       <c r="C200" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B199))</f>
-        <v>0x3FCA3BC8</v>
+        <v>0x3FCA3BC0</v>
       </c>
     </row>
     <row r="201" spans="1:5" x14ac:dyDescent="0.2">
@@ -36611,7 +36721,7 @@
       </c>
       <c r="C201" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B200))</f>
-        <v>0x3FCA3EF4</v>
+        <v>0x3FCA3EEC</v>
       </c>
     </row>
     <row r="202" spans="1:5" x14ac:dyDescent="0.2">
@@ -36623,7 +36733,7 @@
       </c>
       <c r="C202" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B201))</f>
-        <v>0x3FCA3F14</v>
+        <v>0x3FCA3F0C</v>
       </c>
     </row>
     <row r="203" spans="1:5" x14ac:dyDescent="0.2">
@@ -36635,7 +36745,7 @@
       </c>
       <c r="C203" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B202))</f>
-        <v>0x3FCA3F54</v>
+        <v>0x3FCA3F4C</v>
       </c>
     </row>
     <row r="204" spans="1:5" x14ac:dyDescent="0.2">
@@ -36647,16 +36757,16 @@
       </c>
       <c r="C204" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B203))</f>
-        <v>0x3FCA3F58</v>
+        <v>0x3FCA3F50</v>
       </c>
     </row>
     <row r="205" spans="1:5" x14ac:dyDescent="0.2">
       <c r="C205" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B204))</f>
-        <v>0x3FCA3FE8</v>
+        <v>0x3FCA3FE0</v>
       </c>
       <c r="D205" s="8">
-        <f>SUM(B$2:$B205)</f>
+        <f>SUM(B$2:$B204)</f>
         <v>112688</v>
       </c>
       <c r="E205" s="9" t="str">
@@ -36739,7 +36849,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>2542</v>
+        <v>2541</v>
       </c>
       <c r="B7">
         <v>52</v>
@@ -36823,7 +36933,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>2543</v>
+        <v>2542</v>
       </c>
       <c r="B14">
         <v>56</v>
@@ -36859,7 +36969,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>2544</v>
+        <v>2543</v>
       </c>
       <c r="B17">
         <v>48</v>
@@ -37051,7 +37161,7 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>2545</v>
+        <v>2544</v>
       </c>
       <c r="B33">
         <v>12</v>
@@ -37183,7 +37293,7 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>2546</v>
+        <v>2545</v>
       </c>
       <c r="B44">
         <v>164</v>
@@ -37363,7 +37473,7 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>2546</v>
+        <v>2545</v>
       </c>
       <c r="B59">
         <v>516</v>
@@ -37399,7 +37509,7 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>2546</v>
+        <v>2545</v>
       </c>
       <c r="B62">
         <v>16</v>
@@ -37435,7 +37545,7 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>2546</v>
+        <v>2545</v>
       </c>
       <c r="B65">
         <v>84</v>
@@ -37519,7 +37629,7 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>2546</v>
+        <v>2545</v>
       </c>
       <c r="B72">
         <v>592</v>
@@ -37543,7 +37653,7 @@
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>2546</v>
+        <v>2545</v>
       </c>
       <c r="B74" s="2">
         <v>172</v>
@@ -37567,7 +37677,7 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>2546</v>
+        <v>2545</v>
       </c>
       <c r="B76" s="2">
         <v>12</v>
@@ -37639,7 +37749,7 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>2547</v>
+        <v>2546</v>
       </c>
       <c r="B82" s="2">
         <v>4</v>
@@ -37773,7 +37883,7 @@
     <col min="1" max="1" width="71" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>626</v>
       </c>
@@ -37781,7 +37891,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>627</v>
       </c>
@@ -37789,7 +37899,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>628</v>
       </c>
@@ -37797,15 +37907,18 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>629</v>
       </c>
       <c r="B4">
         <v>270</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C4">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>630</v>
       </c>
@@ -37813,23 +37926,29 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>636</v>
       </c>
       <c r="B7">
         <v>22</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C7">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>2548</v>
+        <v>2547</v>
       </c>
       <c r="B8">
         <v>508</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D8">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>633</v>
       </c>
@@ -37837,7 +37956,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>635</v>
       </c>
@@ -37845,7 +37964,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>634</v>
       </c>
@@ -37853,7 +37972,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>637</v>
       </c>
@@ -37861,7 +37980,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>639</v>
       </c>
@@ -37869,7 +37988,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>638</v>
       </c>
@@ -37877,12 +37996,12 @@
         <v>56</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>647</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>646</v>
       </c>
@@ -37890,12 +38009,12 @@
         <v>64</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>644</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>645</v>
       </c>
@@ -37903,20 +38022,23 @@
         <v>58</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>642</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>643</v>
       </c>
       <c r="B22">
         <v>116</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C22">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>641</v>
       </c>
@@ -37924,28 +38046,34 @@
         <v>50</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>640</v>
       </c>
       <c r="B24">
         <v>506</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C24">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>648</v>
       </c>
       <c r="B25">
         <v>508</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C25">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>649</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>650</v>
       </c>
@@ -37953,12 +38081,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>649</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>651</v>
       </c>
@@ -37966,12 +38094,12 @@
         <v>58</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>649</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>652</v>
       </c>
@@ -37979,23 +38107,26 @@
         <v>18</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>2492</v>
       </c>
       <c r="B34">
         <v>972</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C34">
+        <v>990</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>2571</v>
+        <v>2570</v>
       </c>
       <c r="B35">
         <v>72</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>2493</v>
       </c>
@@ -38003,15 +38134,18 @@
         <v>222</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>2494</v>
       </c>
       <c r="B37">
         <v>440</v>
       </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C37">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>2495</v>
       </c>
@@ -38019,15 +38153,18 @@
         <v>110</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>2496</v>
       </c>
       <c r="B39">
         <v>298</v>
       </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C39" s="25" t="s">
+        <v>2580</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>2497</v>
       </c>
@@ -38035,7 +38172,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>2498</v>
       </c>
@@ -38043,7 +38180,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>2499</v>
       </c>
@@ -38051,7 +38188,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>2500</v>
       </c>
@@ -38059,7 +38196,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>2501</v>
       </c>
@@ -38067,7 +38204,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>2472</v>
       </c>
@@ -38075,7 +38212,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>2502</v>
       </c>
@@ -38083,12 +38220,15 @@
         <v>444</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
       <c r="B47">
         <v>630</v>
+      </c>
+      <c r="C47">
+        <v>666</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
@@ -38125,7 +38265,7 @@
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>2574</v>
+        <v>2573</v>
       </c>
       <c r="B53">
         <v>60</v>
@@ -38188,12 +38328,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>2480</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>2481</v>
       </c>
@@ -38201,7 +38341,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>2482</v>
       </c>
@@ -38209,31 +38349,34 @@
         <v>24</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>659</v>
       </c>
       <c r="B68">
         <v>126</v>
       </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C68" s="25"/>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>2478</v>
       </c>
       <c r="B69">
         <v>20</v>
       </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C69" s="25"/>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>653</v>
       </c>
       <c r="B71">
         <v>226</v>
       </c>
-    </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C71" s="25"/>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>653</v>
       </c>
@@ -38241,7 +38384,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>653</v>
       </c>
@@ -38249,7 +38392,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>657</v>
       </c>
@@ -38257,7 +38400,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>658</v>
       </c>
@@ -38265,27 +38408,27 @@
         <v>18</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>631</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>2550</v>
+        <v>2549</v>
       </c>
       <c r="B78">
         <v>28</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>632</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>2551</v>
+        <v>2550</v>
       </c>
       <c r="B80">
         <v>22</v>
@@ -38319,7 +38462,7 @@
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>2573</v>
+        <v>2572</v>
       </c>
       <c r="B86">
         <v>120</v>

</xml_diff>

<commit_message>
Eliminating esp-config (using the current version from crates.io) and rename it to *.me.
It was used by esp-backtrace, esp-embassy, esp-hal and esp-wifi crates. To build my old
crates using esp-config, I had to throw out my old and dirty configuration shortcuts from
build.rs files and start using esp-config.yml configuration files in that crates.

This also brings the whole esp-metadata infrastructure in to the picture, so finally I had to
understand that too (bugajakab stuff, somni language/expressions, etc).

There are many divergent codes in the current libraries: espressif developed its own rtos
library, a minimal embassy like OS for its wifi. It can also be extended/interfaced with embassy.
Esp-hal-embassy crate was replaced by that esp-rtos. Esp-wifi crate was also renamed and migrated
to esp-radio crate using that new OS/runtime crate.
</commit_message>
<xml_diff>
--- a/studies/ecu-via-elm327/sizing.xlsx
+++ b/studies/ecu-via-elm327/sizing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/piv/esp/ccm-diag/studies/ecu-via-elm327/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6546CABF-ECE8-534B-8B36-3A424378893E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDA07865-5F5A-314F-B61A-0D3DCB559E5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="80" yWindow="500" windowWidth="25520" windowHeight="14900" xr2:uid="{7B075F7D-2CA4-8A4E-BD0B-AF2636EE3FAE}"/>
+    <workbookView xWindow="80" yWindow="500" windowWidth="25520" windowHeight="14900" activeTab="9" xr2:uid="{7B075F7D-2CA4-8A4E-BD0B-AF2636EE3FAE}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="11" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2971" uniqueCount="2591">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2973" uniqueCount="2592">
   <si>
     <t>.bss</t>
   </si>
@@ -7796,34 +7796,37 @@
     <t>----</t>
   </si>
   <si>
-    <t>---</t>
-  </si>
-  <si>
     <t>-----</t>
   </si>
   <si>
     <t>x----</t>
   </si>
   <si>
+    <t>x--54</t>
+  </si>
+  <si>
+    <t>x--5b8</t>
+  </si>
+  <si>
+    <t>x++</t>
+  </si>
+  <si>
+    <t>x--66d2</t>
+  </si>
+  <si>
     <t>x--2374</t>
   </si>
   <si>
     <t>x++1062</t>
   </si>
   <si>
-    <t>x--54</t>
-  </si>
-  <si>
-    <t>x++36d4</t>
-  </si>
-  <si>
-    <t>x++66d2</t>
-  </si>
-  <si>
-    <t>x--5b8</t>
+    <t>x++36fc</t>
   </si>
   <si>
     <t>x++3304</t>
+  </si>
+  <si>
+    <t>because embassy_sync changed</t>
   </si>
 </sst>
 </file>
@@ -8472,7 +8475,7 @@
         <v>0x3580</v>
       </c>
       <c r="D8" t="s">
-        <v>2510</v>
+        <v>2585</v>
       </c>
       <c r="F8" t="s">
         <v>2392</v>
@@ -8572,7 +8575,7 @@
         <v>2562</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>2583</v>
+        <v>2582</v>
       </c>
       <c r="F13" t="s">
         <v>2385</v>
@@ -8595,7 +8598,7 @@
         <v>9184</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>2584</v>
+        <v>2587</v>
       </c>
       <c r="F14" t="s">
         <v>2386</v>
@@ -8614,7 +8617,7 @@
         <v>0x1024</v>
       </c>
       <c r="E15" t="s">
-        <v>2585</v>
+        <v>2588</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
@@ -8668,7 +8671,7 @@
         <v>2032</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>2586</v>
+        <v>2583</v>
       </c>
       <c r="F18" t="s">
         <v>2388</v>
@@ -8691,7 +8694,7 @@
         <v>13808</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>2587</v>
+        <v>2589</v>
       </c>
       <c r="F19" t="s">
         <v>2389</v>
@@ -8814,7 +8817,7 @@
         <v>26398</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>2588</v>
+        <v>2586</v>
       </c>
       <c r="F26" t="s">
         <v>2391</v>
@@ -8840,7 +8843,7 @@
         <v>2510</v>
       </c>
       <c r="E27" t="s">
-        <v>2589</v>
+        <v>2584</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
@@ -9179,8 +9182,8 @@
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B28))</f>
         <v>0x420146D6</v>
       </c>
-      <c r="D29" s="25" t="s">
-        <v>2581</v>
+      <c r="D29" s="25">
+        <v>206</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
@@ -9194,8 +9197,8 @@
         <f>"0x"&amp;DEC2HEX(HEX2DEC($C$2)+SUM(B$2:$B29))</f>
         <v>0x420146DE</v>
       </c>
-      <c r="D30" s="25" t="s">
-        <v>2580</v>
+      <c r="D30" s="25">
+        <v>200</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
@@ -10068,7 +10071,7 @@
         <v>0x42015B2C</v>
       </c>
       <c r="D107" s="25" t="s">
-        <v>2582</v>
+        <v>2581</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.2">
@@ -38688,7 +38691,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B33" t="s">
         <v>2461</v>
       </c>
@@ -38696,7 +38699,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B35" t="s">
         <v>2490</v>
       </c>
@@ -38704,7 +38707,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B36" t="s">
         <v>2490</v>
       </c>
@@ -38712,38 +38715,50 @@
         <v>178</v>
       </c>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B37" t="s">
         <v>2490</v>
       </c>
       <c r="C37">
         <v>300</v>
       </c>
-    </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="D37" t="s">
+        <v>2510</v>
+      </c>
+      <c r="E37" t="s">
+        <v>2591</v>
+      </c>
+    </row>
+    <row r="39" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B39" t="s">
         <v>2491</v>
       </c>
       <c r="C39">
         <v>348</v>
       </c>
-    </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="D39" t="s">
+        <v>2510</v>
+      </c>
+      <c r="E39" t="s">
+        <v>2591</v>
+      </c>
+    </row>
+    <row r="41" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B41" t="s">
         <v>2485</v>
       </c>
     </row>
-    <row r="42" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B42" t="s">
         <v>2486</v>
       </c>
     </row>
-    <row r="43" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B43" t="s">
         <v>2487</v>
       </c>
     </row>
-    <row r="44" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="44" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B44" t="s">
         <v>2488</v>
       </c>
@@ -38751,7 +38766,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="45" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="45" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B45" t="s">
         <v>2484</v>
       </c>
@@ -38759,7 +38774,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="46" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="46" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B46" t="s">
         <v>2483</v>
       </c>
@@ -38767,7 +38782,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="48" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B48" t="s">
         <v>679</v>
       </c>

</xml_diff>

<commit_message>
Eliminating esp-backtrace. I've reviewed it carefully again, even the extensa part as well.
I've forked esp-hal and modify esp-backtrace with a patch which eliminate to use println feature.

Then I set patches in config.toml for esp-backtrace and all other crates which were coverged back
to their crates.io version before this commit (esp-println, esp-sync, esp-metadata-generated and
esp-config)i to my forked version of esp-hal.

The defmt feature has limited use here, as it gives the location (PanicInfo) where defmt::panic
calls core::panic!(). So defmt::panic does not give the location info of the original panic.
Therefore, it does not need the core formatting snippets.
I previously posted an issue on https://github.com/knurling-rs/defmt. But now I realized that it
was wrong. The problem is not with the captured addresses -- thay are good -- but this missing
original PanicInfo.
</commit_message>
<xml_diff>
--- a/studies/ecu-via-elm327/sizing.xlsx
+++ b/studies/ecu-via-elm327/sizing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/piv/esp/ccm-diag/studies/ecu-via-elm327/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDA07865-5F5A-314F-B61A-0D3DCB559E5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{355784E7-7E15-A446-ACA0-89C28EF91DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="80" yWindow="500" windowWidth="25520" windowHeight="14900" activeTab="9" xr2:uid="{7B075F7D-2CA4-8A4E-BD0B-AF2636EE3FAE}"/>
+    <workbookView xWindow="80" yWindow="500" windowWidth="25520" windowHeight="14900" xr2:uid="{7B075F7D-2CA4-8A4E-BD0B-AF2636EE3FAE}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="11" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2973" uniqueCount="2592">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2974" uniqueCount="2593">
   <si>
     <t>.bss</t>
   </si>
@@ -7802,31 +7802,34 @@
     <t>x----</t>
   </si>
   <si>
-    <t>x--54</t>
-  </si>
-  <si>
     <t>x--5b8</t>
   </si>
   <si>
     <t>x++</t>
   </si>
   <si>
-    <t>x--66d2</t>
-  </si>
-  <si>
-    <t>x--2374</t>
-  </si>
-  <si>
-    <t>x++1062</t>
-  </si>
-  <si>
-    <t>x++36fc</t>
-  </si>
-  <si>
-    <t>x++3304</t>
-  </si>
-  <si>
     <t>because embassy_sync changed</t>
+  </si>
+  <si>
+    <t>x---f7a</t>
+  </si>
+  <si>
+    <t>x---73c</t>
+  </si>
+  <si>
+    <t>x++3722</t>
+  </si>
+  <si>
+    <t>x+++673c</t>
+  </si>
+  <si>
+    <t>x---54</t>
+  </si>
+  <si>
+    <t>x---2368</t>
+  </si>
+  <si>
+    <t>x++3290</t>
   </si>
 </sst>
 </file>
@@ -8475,7 +8478,7 @@
         <v>0x3580</v>
       </c>
       <c r="D8" t="s">
-        <v>2585</v>
+        <v>2584</v>
       </c>
       <c r="F8" t="s">
         <v>2392</v>
@@ -8598,7 +8601,7 @@
         <v>9184</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>2587</v>
+        <v>2591</v>
       </c>
       <c r="F14" t="s">
         <v>2386</v>
@@ -8617,7 +8620,7 @@
         <v>0x1024</v>
       </c>
       <c r="E15" t="s">
-        <v>2588</v>
+        <v>2586</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
@@ -8653,6 +8656,9 @@
         <f t="shared" si="1"/>
         <v>0x754</v>
       </c>
+      <c r="E17" s="6" t="s">
+        <v>2587</v>
+      </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
@@ -8671,7 +8677,7 @@
         <v>2032</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>2583</v>
+        <v>2590</v>
       </c>
       <c r="F18" t="s">
         <v>2388</v>
@@ -8694,7 +8700,7 @@
         <v>13808</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>2589</v>
+        <v>2588</v>
       </c>
       <c r="F19" t="s">
         <v>2389</v>
@@ -8817,7 +8823,7 @@
         <v>26398</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>2586</v>
+        <v>2589</v>
       </c>
       <c r="F26" t="s">
         <v>2391</v>
@@ -8843,7 +8849,7 @@
         <v>2510</v>
       </c>
       <c r="E27" t="s">
-        <v>2584</v>
+        <v>2583</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
@@ -8862,7 +8868,7 @@
         <v>2510</v>
       </c>
       <c r="E28" t="s">
-        <v>2590</v>
+        <v>2592</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
@@ -38726,7 +38732,7 @@
         <v>2510</v>
       </c>
       <c r="E37" t="s">
-        <v>2591</v>
+        <v>2585</v>
       </c>
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.2">
@@ -38740,7 +38746,7 @@
         <v>2510</v>
       </c>
       <c r="E39" t="s">
-        <v>2591</v>
+        <v>2585</v>
       </c>
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Rename riscv (riscv, riscv-rt, rsicv-pac). Reviewing and using the new versions from crates.io.
It nedded some modification in esp-hal, since riscv's register API had changed a bit.
</commit_message>
<xml_diff>
--- a/studies/ecu-via-elm327/sizing.xlsx
+++ b/studies/ecu-via-elm327/sizing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/piv/esp/ccm-diag/studies/ecu-via-elm327/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{355784E7-7E15-A446-ACA0-89C28EF91DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81B7B36A-77CB-284B-912D-792AE489D83F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="80" yWindow="500" windowWidth="25520" windowHeight="14900" xr2:uid="{7B075F7D-2CA4-8A4E-BD0B-AF2636EE3FAE}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2974" uniqueCount="2593">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2972" uniqueCount="2592">
   <si>
     <t>.bss</t>
   </si>
@@ -7775,9 +7775,6 @@
     <t>esp_hal::gpio::PinGuard as core::ops::drop::Drop::drop</t>
   </si>
   <si>
-    <t>42058abc</t>
-  </si>
-  <si>
     <t>if we change" inline"to "inline(always)" of this function in core::slice, this shrinks to 2 bytes</t>
   </si>
   <si>
@@ -7802,34 +7799,34 @@
     <t>x----</t>
   </si>
   <si>
-    <t>x--5b8</t>
-  </si>
-  <si>
-    <t>x++</t>
-  </si>
-  <si>
     <t>because embassy_sync changed</t>
   </si>
   <si>
-    <t>x---f7a</t>
-  </si>
-  <si>
-    <t>x---73c</t>
-  </si>
-  <si>
-    <t>x++3722</t>
-  </si>
-  <si>
-    <t>x+++673c</t>
-  </si>
-  <si>
     <t>x---54</t>
   </si>
   <si>
-    <t>x---2368</t>
-  </si>
-  <si>
-    <t>x++3290</t>
+    <t>x+++1b870</t>
+  </si>
+  <si>
+    <t>x+++3738</t>
+  </si>
+  <si>
+    <t>x---2376</t>
+  </si>
+  <si>
+    <t>x---fa6</t>
+  </si>
+  <si>
+    <t>x---6ac</t>
+  </si>
+  <si>
+    <t>x++337a</t>
+  </si>
+  <si>
+    <t>x+++6770</t>
+  </si>
+  <si>
+    <t>was 64a</t>
   </si>
 </sst>
 </file>
@@ -8394,7 +8391,7 @@
       </c>
       <c r="G4" s="21">
         <f>SUM(B12:B28)+14</f>
-        <v>311272</v>
+        <v>304362</v>
       </c>
       <c r="H4" s="21" t="s">
         <v>2380</v>
@@ -8459,10 +8456,13 @@
         <f t="shared" si="0"/>
         <v>0x1B830</v>
       </c>
+      <c r="D7" t="s">
+        <v>2584</v>
+      </c>
       <c r="F7" s="4"/>
       <c r="G7" s="22">
         <f>G1+G2+G4+G6</f>
-        <v>386024</v>
+        <v>379114</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
@@ -8478,14 +8478,14 @@
         <v>0x3580</v>
       </c>
       <c r="D8" t="s">
-        <v>2584</v>
+        <v>2585</v>
       </c>
       <c r="F8" t="s">
         <v>2392</v>
       </c>
       <c r="G8" s="21">
         <f>G1+G4</f>
-        <v>351288</v>
+        <v>344378</v>
       </c>
       <c r="I8" s="23"/>
     </row>
@@ -8509,7 +8509,7 @@
       </c>
       <c r="H9" s="22">
         <f>G8+G9</f>
-        <v>386024</v>
+        <v>379114</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
@@ -8578,7 +8578,7 @@
         <v>2562</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>2582</v>
+        <v>2581</v>
       </c>
       <c r="F13" t="s">
         <v>2385</v>
@@ -8601,7 +8601,7 @@
         <v>9184</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>2591</v>
+        <v>2586</v>
       </c>
       <c r="F14" t="s">
         <v>2386</v>
@@ -8620,7 +8620,7 @@
         <v>0x1024</v>
       </c>
       <c r="E15" t="s">
-        <v>2586</v>
+        <v>2587</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
@@ -8657,7 +8657,7 @@
         <v>0x754</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>2587</v>
+        <v>2588</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
@@ -8677,7 +8677,7 @@
         <v>2032</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>2590</v>
+        <v>2583</v>
       </c>
       <c r="F18" t="s">
         <v>2388</v>
@@ -8700,7 +8700,7 @@
         <v>13808</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>2588</v>
+        <v>2589</v>
       </c>
       <c r="F19" t="s">
         <v>2389</v>
@@ -8772,10 +8772,10 @@
       </c>
       <c r="G24" s="21">
         <f>D13+D14+D16+D18+D19+D25+D26+B27+B28+14</f>
-        <v>341020</v>
+        <v>334110</v>
       </c>
       <c r="H24" s="21" t="s">
-        <v>2577</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
@@ -8803,7 +8803,7 @@
         <v>45004</v>
       </c>
       <c r="H25" s="21" t="s">
-        <v>2578</v>
+        <v>2577</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
@@ -8823,14 +8823,14 @@
         <v>26398</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>2589</v>
+        <v>2590</v>
       </c>
       <c r="F26" t="s">
         <v>2391</v>
       </c>
       <c r="G26" s="21">
         <f>G24+G25</f>
-        <v>386024</v>
+        <v>379114</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
@@ -8838,18 +8838,18 @@
         <v>607</v>
       </c>
       <c r="B27" s="6">
-        <f>'core-text'!D26</f>
-        <v>1610</v>
+        <f>'core-text'!D25</f>
+        <v>1464</v>
       </c>
       <c r="C27" s="10" t="str">
         <f t="shared" si="1"/>
-        <v>0x64A</v>
+        <v>0x5B8</v>
       </c>
       <c r="D27" t="s">
         <v>2510</v>
       </c>
       <c r="E27" t="s">
-        <v>2583</v>
+        <v>2591</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
@@ -8857,18 +8857,15 @@
         <v>608</v>
       </c>
       <c r="B28" s="6">
-        <f>'core-text'!D47</f>
-        <v>12030</v>
+        <f>'core-text'!D46</f>
+        <v>5266</v>
       </c>
       <c r="C28" s="10" t="str">
         <f t="shared" si="1"/>
-        <v>0x2EFE</v>
+        <v>0x1492</v>
       </c>
       <c r="D28" t="s">
         <v>2510</v>
-      </c>
-      <c r="E28" t="s">
-        <v>2592</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
@@ -10077,7 +10074,7 @@
         <v>0x42015B2C</v>
       </c>
       <c r="D107" s="25" t="s">
-        <v>2581</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.2">
@@ -29363,7 +29360,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA0F76B8-C396-BD43-B16C-9B2C32D8D617}">
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="53.33203125" customWidth="1"/>
@@ -29382,14 +29379,14 @@
       <c r="C2">
         <v>24</v>
       </c>
-      <c r="D2" s="10" t="s">
-        <v>2574</v>
+      <c r="D2" s="10">
+        <v>42058548</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="D3" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C2))</f>
-        <v>0x42058AD4</v>
+        <v>0x42058560</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -29401,7 +29398,7 @@
       </c>
       <c r="D4" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C3))</f>
-        <v>0x42058AD4</v>
+        <v>0x42058560</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -29413,7 +29410,7 @@
       </c>
       <c r="D5" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C4))</f>
-        <v>0x42058AD6</v>
+        <v>0x42058562</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -29425,7 +29422,7 @@
       </c>
       <c r="D6" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C5))</f>
-        <v>0x42058B38</v>
+        <v>0x420585C4</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -29437,7 +29434,7 @@
       </c>
       <c r="D7" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C6))</f>
-        <v>0x42058BCC</v>
+        <v>0x42058658</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -29449,13 +29446,13 @@
       </c>
       <c r="D8" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C7))</f>
-        <v>0x42058BCE</v>
+        <v>0x4205865A</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="D9" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C8))</f>
-        <v>0x42058C66</v>
+        <v>0x420586F2</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -29467,13 +29464,13 @@
       </c>
       <c r="D10" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C9))</f>
-        <v>0x42058C66</v>
+        <v>0x420586F2</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="D11" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C10))</f>
-        <v>0x42058C82</v>
+        <v>0x4205870E</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -29482,7 +29479,7 @@
       </c>
       <c r="D12" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C11))</f>
-        <v>0x42058C82</v>
+        <v>0x4205870E</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
@@ -29494,7 +29491,7 @@
       </c>
       <c r="D13" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C12))</f>
-        <v>0x42058C82</v>
+        <v>0x4205870E</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
@@ -29506,137 +29503,136 @@
       </c>
       <c r="D14" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C13))</f>
-        <v>0x42058CD0</v>
+        <v>0x4205875C</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
-        <v>2489</v>
-      </c>
-      <c r="C15">
-        <v>146</v>
+        <v>2373</v>
       </c>
       <c r="D15" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C14))</f>
-        <v>0x42058DB0</v>
+        <v>0x4205883C</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
-        <v>2373</v>
+        <v>2374</v>
       </c>
       <c r="D16" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C15))</f>
-        <v>0x42058E42</v>
+        <v>0x4205883C</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
-        <v>2374</v>
+        <v>2553</v>
       </c>
       <c r="D17" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C16))</f>
-        <v>0x42058E42</v>
+        <v>0x4205883C</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
-        <v>2553</v>
+        <v>2554</v>
+      </c>
+      <c r="C18">
+        <v>2</v>
       </c>
       <c r="D18" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C17))</f>
-        <v>0x42058E42</v>
+        <v>0x4205883C</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B19" t="s">
-        <v>2554</v>
-      </c>
-      <c r="C19">
-        <v>2</v>
-      </c>
       <c r="D19" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C18))</f>
-        <v>0x42058E42</v>
+        <v>0x4205883E</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B20" t="s">
+        <v>2555</v>
+      </c>
+      <c r="C20">
+        <f>11*62+20</f>
+        <v>702</v>
+      </c>
       <c r="D20" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C19))</f>
-        <v>0x42058E44</v>
+        <v>0x4205883E</v>
+      </c>
+      <c r="F20" t="s">
+        <v>2574</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B21" t="s">
-        <v>2555</v>
-      </c>
-      <c r="C21">
-        <f>11*62+20</f>
-        <v>702</v>
-      </c>
       <c r="D21" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C20))</f>
-        <v>0x42058E44</v>
+        <v>0x42058AFC</v>
       </c>
       <c r="F21" t="s">
         <v>2575</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>2556</v>
+      </c>
+      <c r="C22">
+        <v>2</v>
+      </c>
       <c r="D22" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C21))</f>
-        <v>0x42059102</v>
-      </c>
-      <c r="F22" t="s">
-        <v>2576</v>
+        <v>0x42058AFC</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
-        <v>2556</v>
-      </c>
-      <c r="C23">
-        <v>2</v>
+        <v>2449</v>
       </c>
       <c r="D23" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C22))</f>
-        <v>0x42059102</v>
+        <v>0x42058AFE</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
-        <v>2449</v>
+        <v>2450</v>
+      </c>
+      <c r="C24">
+        <v>2</v>
       </c>
       <c r="D24" s="11" t="str">
         <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C23))</f>
-        <v>0x42059104</v>
+        <v>0x42058AFE</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B25" t="s">
-        <v>2450</v>
-      </c>
-      <c r="C25">
-        <v>2</v>
-      </c>
-      <c r="D25" s="11" t="str">
-        <f>"0x"&amp;DEC2HEX(HEX2DEC($D$2)+SUM($C$2:C24))</f>
-        <v>0x42059104</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="D26" s="20">
-        <f>SUM(C2:$C$25)</f>
-        <v>1610</v>
-      </c>
-      <c r="E26" s="9" t="str">
-        <f>"0x"&amp;DEC2HEX(D26)</f>
-        <v>0x64A</v>
+      <c r="D25" s="20">
+        <f>SUM(C2:$C$24)</f>
+        <v>1464</v>
+      </c>
+      <c r="E25" s="9" t="str">
+        <f>"0x"&amp;DEC2HEX(D25)</f>
+        <v>0x5B8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>608</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>608</v>
+      <c r="B28" t="s">
+        <v>548</v>
+      </c>
+      <c r="C28">
+        <v>6764</v>
+      </c>
+      <c r="D28" s="10">
+        <v>6908</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
@@ -29647,7 +29643,7 @@
         <v>1924</v>
       </c>
       <c r="D29" s="10">
-        <v>1952</v>
+        <v>1990</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
@@ -29655,10 +29651,10 @@
         <v>548</v>
       </c>
       <c r="C30">
-        <v>6764</v>
+        <v>1398</v>
       </c>
       <c r="D30" s="10">
-        <v>6908</v>
+        <v>1426</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
@@ -29666,10 +29662,10 @@
         <v>548</v>
       </c>
       <c r="C31">
-        <v>146</v>
+        <v>108</v>
       </c>
       <c r="D31" s="10">
-        <v>212</v>
+        <v>110</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
@@ -29677,99 +29673,97 @@
         <v>548</v>
       </c>
       <c r="C32">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B33" t="s">
-        <v>548</v>
-      </c>
-      <c r="C33">
-        <v>1398</v>
-      </c>
-      <c r="D33" s="10">
-        <v>1412</v>
+        <v>146</v>
+      </c>
+      <c r="D32" s="10">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B34" t="s">
+        <v>2557</v>
       </c>
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B35" t="s">
-        <v>2557</v>
+        <v>2558</v>
+      </c>
+      <c r="C35">
+        <v>464</v>
+      </c>
+      <c r="D35" s="10">
+        <v>506</v>
       </c>
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B36" t="s">
-        <v>2558</v>
-      </c>
-      <c r="C36">
-        <v>464</v>
+        <v>2557</v>
       </c>
     </row>
     <row r="37" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B37" t="s">
-        <v>2557</v>
+        <v>2559</v>
+      </c>
+      <c r="C37">
+        <v>312</v>
       </c>
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B38" t="s">
-        <v>2559</v>
-      </c>
-      <c r="C38">
-        <v>312</v>
+        <v>2557</v>
       </c>
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B39" t="s">
-        <v>2557</v>
+        <v>2560</v>
+      </c>
+      <c r="C39">
+        <v>282</v>
+      </c>
+      <c r="D39" s="10">
+        <v>530</v>
       </c>
     </row>
     <row r="40" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B40" t="s">
-        <v>2560</v>
+        <v>2561</v>
       </c>
       <c r="C40">
-        <v>282</v>
+        <v>314</v>
       </c>
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B41" t="s">
-        <v>2561</v>
+        <v>2562</v>
       </c>
       <c r="C41">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="42" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B42" t="s">
-        <v>2562</v>
-      </c>
-      <c r="C42">
         <v>300</v>
       </c>
     </row>
-    <row r="44" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B44" t="s">
+    <row r="43" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B43" t="s">
         <v>2571</v>
       </c>
-      <c r="C44">
+      <c r="C43">
         <v>2</v>
       </c>
     </row>
+    <row r="45" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B45" t="s">
+        <v>2376</v>
+      </c>
+      <c r="C45">
+        <v>16</v>
+      </c>
+    </row>
     <row r="46" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B46" t="s">
-        <v>2376</v>
-      </c>
-      <c r="C46">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="47" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="D47" s="20">
-        <f>SUM(C$29:$C46)</f>
-        <v>12030</v>
-      </c>
-      <c r="E47" s="9" t="str">
-        <f>"0x"&amp;DEC2HEX(D47)</f>
-        <v>0x2EFE</v>
+      <c r="D46" s="20">
+        <f>SUM(C$29:$C45)</f>
+        <v>5266</v>
+      </c>
+      <c r="E46" s="9" t="str">
+        <f>"0x"&amp;DEC2HEX(D46)</f>
+        <v>0x1492</v>
       </c>
     </row>
   </sheetData>
@@ -34366,7 +34360,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>2579</v>
+        <v>2578</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -38170,7 +38164,7 @@
         <v>298</v>
       </c>
       <c r="C39" s="25" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
@@ -38732,7 +38726,7 @@
         <v>2510</v>
       </c>
       <c r="E37" t="s">
-        <v>2585</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.2">
@@ -38746,7 +38740,7 @@
         <v>2510</v>
       </c>
       <c r="E39" t="s">
-        <v>2585</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Testing our esp-radio/no_wap_supplicant feature. Code and RAM savings in sizing.xlsx
If use only AP in wifi communication, we can skip esp_supplicant_init in esp-radio crate.
It saves 35K code and 1K RAM space.
</commit_message>
<xml_diff>
--- a/studies/ecu-via-elm327/sizing.xlsx
+++ b/studies/ecu-via-elm327/sizing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/piv/esp/ccm-diag/studies/ecu-via-elm327/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E81859C-EC25-C145-B9EE-165AC2788BB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2961A086-5FEB-9947-A4AA-4712BEDB9388}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="80" yWindow="500" windowWidth="25520" windowHeight="14900" activeTab="1" xr2:uid="{7B075F7D-2CA4-8A4E-BD0B-AF2636EE3FAE}"/>
+    <workbookView xWindow="80" yWindow="500" windowWidth="25520" windowHeight="14900" xr2:uid="{7B075F7D-2CA4-8A4E-BD0B-AF2636EE3FAE}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="11" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3340" uniqueCount="2812">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3366" uniqueCount="2823">
   <si>
     <t>.bss</t>
   </si>
@@ -8489,6 +8489,39 @@
   </si>
   <si>
     <t>esp_hal::system::assert_peri_reset_racey (match statement)</t>
+  </si>
+  <si>
+    <t>Updated in this commit</t>
+  </si>
+  <si>
+    <t>if esp-radio/no_wap_supplicant feature</t>
+  </si>
+  <si>
+    <t>-&gt;</t>
+  </si>
+  <si>
+    <t>0xC2D0</t>
+  </si>
+  <si>
+    <t>0x2D2C</t>
+  </si>
+  <si>
+    <t>0x6F54</t>
+  </si>
+  <si>
+    <t>0x1edc</t>
+  </si>
+  <si>
+    <t>0x1f5bc</t>
+  </si>
+  <si>
+    <t>0x3fda</t>
+  </si>
+  <si>
+    <t>0x284</t>
+  </si>
+  <si>
+    <t>0x5250</t>
   </si>
 </sst>
 </file>
@@ -8589,7 +8622,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -8636,6 +8669,12 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8950,7 +8989,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37E27708-F997-1741-9963-F7C4C3F90832}">
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
@@ -9423,7 +9462,7 @@
         <v>39676</v>
       </c>
       <c r="C24" s="9" t="str">
-        <f t="shared" si="1"/>
+        <f>"0x"&amp;DEC2HEX(B24)</f>
         <v>0x9AFC</v>
       </c>
     </row>
@@ -9574,6 +9613,194 @@
         <v>347586</v>
       </c>
       <c r="E31" s="18"/>
+      <c r="F31" t="s">
+        <v>2812</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>2813</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>0</v>
+      </c>
+      <c r="B34" s="18">
+        <f>B7</f>
+        <v>50832</v>
+      </c>
+      <c r="C34" s="9" t="str">
+        <f t="shared" ref="C34:C37" si="2">"0x"&amp;DEC2HEX(B34)</f>
+        <v>0xC690</v>
+      </c>
+      <c r="D34" s="26" t="s">
+        <v>2814</v>
+      </c>
+      <c r="E34" t="s">
+        <v>2815</v>
+      </c>
+      <c r="F34" s="27">
+        <v>-960</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>1</v>
+      </c>
+      <c r="B35" s="18">
+        <f>B8</f>
+        <v>11748</v>
+      </c>
+      <c r="C35" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v>0x2DE4</v>
+      </c>
+      <c r="D35" s="26" t="s">
+        <v>2814</v>
+      </c>
+      <c r="E35" t="s">
+        <v>2816</v>
+      </c>
+      <c r="F35" s="27">
+        <v>-184</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>2011</v>
+      </c>
+      <c r="B36" s="18">
+        <f>B9</f>
+        <v>29204</v>
+      </c>
+      <c r="C36" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v>0x7214</v>
+      </c>
+      <c r="D36" s="26" t="s">
+        <v>2814</v>
+      </c>
+      <c r="E36" t="s">
+        <v>2817</v>
+      </c>
+      <c r="F36" s="27">
+        <v>-704</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>415</v>
+      </c>
+      <c r="B37" s="18">
+        <f>B17</f>
+        <v>674</v>
+      </c>
+      <c r="C37" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v>0x2A2</v>
+      </c>
+      <c r="D37" s="26" t="s">
+        <v>2814</v>
+      </c>
+      <c r="E37" t="s">
+        <v>2821</v>
+      </c>
+      <c r="F37" s="27">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>2464</v>
+      </c>
+      <c r="B38" s="18">
+        <f>B21</f>
+        <v>7944</v>
+      </c>
+      <c r="C38" s="9" t="str">
+        <f t="shared" ref="C38" si="3">"0x"&amp;DEC2HEX(B38)</f>
+        <v>0x1F08</v>
+      </c>
+      <c r="D38" s="26" t="s">
+        <v>2814</v>
+      </c>
+      <c r="E38" t="s">
+        <v>2818</v>
+      </c>
+      <c r="F38" s="27">
+        <v>-44</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>419</v>
+      </c>
+      <c r="B39" s="18">
+        <f>B26</f>
+        <v>132818</v>
+      </c>
+      <c r="C39" s="9" t="str">
+        <f t="shared" ref="C39" si="4">"0x"&amp;DEC2HEX(B39)</f>
+        <v>0x206D2</v>
+      </c>
+      <c r="D39" s="26" t="s">
+        <v>2814</v>
+      </c>
+      <c r="E39" t="s">
+        <v>2819</v>
+      </c>
+      <c r="F39" s="27">
+        <v>-4374</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>4</v>
+      </c>
+      <c r="B40" s="18">
+        <f>B27</f>
+        <v>46738</v>
+      </c>
+      <c r="C40" s="9" t="str">
+        <f t="shared" ref="C40" si="5">"0x"&amp;DEC2HEX(B40)</f>
+        <v>0xB692</v>
+      </c>
+      <c r="D40" s="26" t="s">
+        <v>2814</v>
+      </c>
+      <c r="E40" t="s">
+        <v>2820</v>
+      </c>
+      <c r="F40" s="27">
+        <v>-30392</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>2774</v>
+      </c>
+      <c r="B41" s="18">
+        <f>B30</f>
+        <v>21102</v>
+      </c>
+      <c r="C41" s="9" t="str">
+        <f t="shared" ref="C41" si="6">"0x"&amp;DEC2HEX(B41)</f>
+        <v>0x526E</v>
+      </c>
+      <c r="D41" s="26" t="s">
+        <v>2814</v>
+      </c>
+      <c r="E41" t="s">
+        <v>2822</v>
+      </c>
+      <c r="F41" s="27">
+        <v>-30</v>
+      </c>
+      <c r="G41" s="18">
+        <f>SUM(F35:F41)</f>
+        <v>-35758</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Putting ssid, ip and port into env variables, a small refactoring of main/loader and udp task
</commit_message>
<xml_diff>
--- a/studies/ecu-via-elm327/sizing.xlsx
+++ b/studies/ecu-via-elm327/sizing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/piv/esp/ccm-diag/studies/ecu-via-elm327/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2961A086-5FEB-9947-A4AA-4712BEDB9388}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CDDEBD3-6219-B74F-B3CB-55BC432D8CDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="80" yWindow="500" windowWidth="25520" windowHeight="14900" xr2:uid="{7B075F7D-2CA4-8A4E-BD0B-AF2636EE3FAE}"/>
   </bookViews>
@@ -8491,9 +8491,6 @@
     <t>esp_hal::system::assert_peri_reset_racey (match statement)</t>
   </si>
   <si>
-    <t>Updated in this commit</t>
-  </si>
-  <si>
     <t>if esp-radio/no_wap_supplicant feature</t>
   </si>
   <si>
@@ -8522,6 +8519,9 @@
   </si>
   <si>
     <t>0x5250</t>
+  </si>
+  <si>
+    <t>Updated not in this commit</t>
   </si>
 </sst>
 </file>
@@ -9614,12 +9614,12 @@
       </c>
       <c r="E31" s="18"/>
       <c r="F31" t="s">
-        <v>2812</v>
+        <v>2822</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>2813</v>
+        <v>2812</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
@@ -9635,10 +9635,10 @@
         <v>0xC690</v>
       </c>
       <c r="D34" s="26" t="s">
+        <v>2813</v>
+      </c>
+      <c r="E34" t="s">
         <v>2814</v>
-      </c>
-      <c r="E34" t="s">
-        <v>2815</v>
       </c>
       <c r="F34" s="27">
         <v>-960</v>
@@ -9657,10 +9657,10 @@
         <v>0x2DE4</v>
       </c>
       <c r="D35" s="26" t="s">
-        <v>2814</v>
+        <v>2813</v>
       </c>
       <c r="E35" t="s">
-        <v>2816</v>
+        <v>2815</v>
       </c>
       <c r="F35" s="27">
         <v>-184</v>
@@ -9679,10 +9679,10 @@
         <v>0x7214</v>
       </c>
       <c r="D36" s="26" t="s">
-        <v>2814</v>
+        <v>2813</v>
       </c>
       <c r="E36" t="s">
-        <v>2817</v>
+        <v>2816</v>
       </c>
       <c r="F36" s="27">
         <v>-704</v>
@@ -9701,10 +9701,10 @@
         <v>0x2A2</v>
       </c>
       <c r="D37" s="26" t="s">
-        <v>2814</v>
+        <v>2813</v>
       </c>
       <c r="E37" t="s">
-        <v>2821</v>
+        <v>2820</v>
       </c>
       <c r="F37" s="27">
         <v>-30</v>
@@ -9723,10 +9723,10 @@
         <v>0x1F08</v>
       </c>
       <c r="D38" s="26" t="s">
-        <v>2814</v>
+        <v>2813</v>
       </c>
       <c r="E38" t="s">
-        <v>2818</v>
+        <v>2817</v>
       </c>
       <c r="F38" s="27">
         <v>-44</v>
@@ -9745,10 +9745,10 @@
         <v>0x206D2</v>
       </c>
       <c r="D39" s="26" t="s">
-        <v>2814</v>
+        <v>2813</v>
       </c>
       <c r="E39" t="s">
-        <v>2819</v>
+        <v>2818</v>
       </c>
       <c r="F39" s="27">
         <v>-4374</v>
@@ -9767,10 +9767,10 @@
         <v>0xB692</v>
       </c>
       <c r="D40" s="26" t="s">
-        <v>2814</v>
+        <v>2813</v>
       </c>
       <c r="E40" t="s">
-        <v>2820</v>
+        <v>2819</v>
       </c>
       <c r="F40" s="27">
         <v>-30392</v>
@@ -9789,10 +9789,10 @@
         <v>0x526E</v>
       </c>
       <c r="D41" s="26" t="s">
-        <v>2814</v>
+        <v>2813</v>
       </c>
       <c r="E41" t="s">
-        <v>2822</v>
+        <v>2821</v>
       </c>
       <c r="F41" s="27">
         <v>-30</v>

</xml_diff>

<commit_message>
Putting ELM327 adapter to specific, and prepare general architecture for ecu, protocol and adapter modules
</commit_message>
<xml_diff>
--- a/studies/ecu-via-elm327/sizing.xlsx
+++ b/studies/ecu-via-elm327/sizing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/piv/esp/ccm-diag/studies/ecu-via-elm327/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{632798BC-B57A-6443-965C-53022E2F9532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA7841E4-E7AC-4B4E-8813-066EF9FD4992}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="80" yWindow="500" windowWidth="25520" windowHeight="14900" xr2:uid="{7B075F7D-2CA4-8A4E-BD0B-AF2636EE3FAE}"/>
   </bookViews>
@@ -7567,13 +7567,13 @@
     <t>ecu_via_elm327::udp::send_to::closure</t>
   </si>
   <si>
-    <t>Updated in this commit</t>
-  </si>
-  <si>
     <t>420277a8</t>
   </si>
   <si>
     <t>embassy_executor::raw::util::UninitCel::write_in_place</t>
+  </si>
+  <si>
+    <t>NOT Updated in this commit</t>
   </si>
 </sst>
 </file>
@@ -8665,7 +8665,7 @@
       </c>
       <c r="E31" s="18"/>
       <c r="F31" t="s">
-        <v>2504</v>
+        <v>2506</v>
       </c>
     </row>
   </sheetData>
@@ -8708,7 +8708,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="C4">
         <v>22</v>
@@ -8720,7 +8720,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="C5">
         <v>6</v>
@@ -8732,7 +8732,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="C6">
         <v>22</v>
@@ -8744,7 +8744,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="C7">
         <v>18</v>
@@ -8756,7 +8756,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="C8">
         <v>8</v>
@@ -19274,7 +19274,7 @@
         <v>948</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>2505</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>